<commit_message>
feat(template): perbaiki template subsistem Suralaya-Cilegon 100% sesuai diagram SLD PLN
</commit_message>
<xml_diff>
--- a/peta-kerawanan/dist/template_kerawanan_subsistem_suralaya_cilegon.xlsx
+++ b/peta-kerawanan/dist/template_kerawanan_subsistem_suralaya_cilegon.xlsx
@@ -400,7 +400,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y21"/>
+  <dimension ref="A1:Y28"/>
+  <cols>
+    <col min="1" max="1" width="5.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" customWidth="1"/>
+    <col min="17" max="17" width="24.83203125" customWidth="1"/>
+    <col min="18" max="18" width="24.83203125" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+    <col min="20" max="20" width="22.83203125" customWidth="1"/>
+    <col min="21" max="21" width="10.83203125" customWidth="1"/>
+    <col min="22" max="22" width="45.83203125" customWidth="1"/>
+    <col min="23" max="23" width="35.83203125" customWidth="1"/>
+    <col min="24" max="24" width="35.83203125" customWidth="1"/>
+    <col min="25" max="25" width="35.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -479,27 +506,27 @@
         <v>Usulan / Solusi</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>1&amp;2</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>Bay IBT 2 Suralaya Baru (500/150 kV)</v>
+        <v>Bay Evakuasi PLTU Suralaya Unit 3</v>
       </c>
       <c r="D2" t="str">
-        <v>Bay IBT</v>
+        <v>Bay Generator &amp; GSUT</v>
       </c>
       <c r="E2" t="str">
-        <v>IBT</v>
+        <v>trafo_generator</v>
       </c>
       <c r="F2" t="str">
-        <v>Suralaya Baru</v>
+        <v>Unit 3</v>
       </c>
       <c r="G2" t="str">
-        <v>Busbar</v>
+        <v>generator</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -508,13 +535,13 @@
         <v>SRLYA</v>
       </c>
       <c r="J2" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="K2">
         <v>1</v>
       </c>
       <c r="L2" t="str">
-        <v>500/150 kV</v>
+        <v>500 kV</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -526,16 +553,16 @@
         <v>Beroperasi</v>
       </c>
       <c r="P2" t="str">
-        <v>Sangat Rawan</v>
+        <v>Normal</v>
       </c>
       <c r="Q2">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="R2" t="str">
         <v/>
       </c>
       <c r="S2">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="T2" t="str">
         <v>Banten - Cilegon</v>
@@ -544,101 +571,98 @@
         <v>JBB</v>
       </c>
       <c r="V2" t="str">
+        <v>Bay Pembangkit Unit 3: 1. Generator (Hijau), 2. Trafo GSUT (Hijau-Merah), 3. CB PMT (Balok Merah)</v>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>1&amp;2</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Bay IBT 2 Suralaya Baru (500/150 kV)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Bay Interbus Transformer</v>
+      </c>
+      <c r="E3" t="str">
+        <v>ibt</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Suralaya Baru</v>
+      </c>
+      <c r="G3" t="str">
+        <v>busbar</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" t="str">
+        <v>SRLYA</v>
+      </c>
+      <c r="J3" t="str">
+        <v>busbar</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3" t="str">
+        <v>500/150 kV</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Beroperasi</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Sangat Rawan</v>
+      </c>
+      <c r="Q3">
+        <v>88</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3">
+        <v>0.5</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Banten - Cilegon</v>
+      </c>
+      <c r="U3" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V3" t="str">
         <v>Pembebanan IBT–1,2 Suralaya tidak memenuhi kriteria N–1 saat PLTU Suralaya unit–3 tidak beroperasi dan IBT–4 Cilegon masuk sub sistem Cilegon.</v>
       </c>
-      <c r="W2" t="str" xml:space="preserve">
+      <c r="W3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Pemeliharaan IBT sulit dilakukan.
 2. Pertumbuhan beban menjadi terhambat.
 3. Terjadi pemadaman apabila trip salah satu IBT di Suralaya.</v>
       </c>
-      <c r="X2" t="str" xml:space="preserve">
+      <c r="X3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW.
-2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan total target sebesar 137 MW.
+2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan target total 137 MW.
 3. Pemeliharaan IBT saat beban rendah.</v>
-      </c>
-      <c r="Y2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2025.</v>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>1&amp;2</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Bay IBT 1 Suralaya (500/150 kV)</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Bay IBT</v>
-      </c>
-      <c r="E3" t="str">
-        <v>IBT</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Suralaya</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Busbar</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3" t="str">
-        <v>SRLYA</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Busbar</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3" t="str">
-        <v>500/150 kV</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-      <c r="N3">
-        <v>1</v>
-      </c>
-      <c r="O3" t="str">
-        <v>Beroperasi</v>
-      </c>
-      <c r="P3" t="str">
-        <v>Sangat Rawan</v>
-      </c>
-      <c r="Q3">
-        <v>84</v>
-      </c>
-      <c r="R3" t="str">
-        <v/>
-      </c>
-      <c r="S3">
-        <v>0.5</v>
-      </c>
-      <c r="T3" t="str">
-        <v>Banten - Cilegon</v>
-      </c>
-      <c r="U3" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="V3" t="str">
-        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA sedangkan IBT #4 Cilegon 500 MVA).</v>
-      </c>
-      <c r="W3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Ketidakseimbangan beban antara IBT Suralaya dan IBT Cilegon.
-2. Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
-      </c>
-      <c r="X3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya.
-2. Pemeliharaan IBT saat beban rendah.</v>
       </c>
       <c r="Y3" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2026.</v>
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD Tahun 2025.</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -646,31 +670,31 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>2</v>
+        <v>1&amp;2</v>
       </c>
       <c r="C4" t="str">
-        <v>Bay IBT 4 Cilegon Baru (500/150 kV)</v>
+        <v>Bay IBT 1 Suralaya (500/150 kV)</v>
       </c>
       <c r="D4" t="str">
-        <v>Bay IBT</v>
+        <v>Bay Interbus Transformer</v>
       </c>
       <c r="E4" t="str">
-        <v>IBT</v>
+        <v>ibt</v>
       </c>
       <c r="F4" t="str">
-        <v>Cilegon Baru</v>
+        <v>Suralaya</v>
       </c>
       <c r="G4" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4" t="str">
-        <v>CLBRU</v>
+        <v>SRLYA</v>
       </c>
       <c r="J4" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="K4">
         <v>1</v>
@@ -691,7 +715,7 @@
         <v>Sangat Rawan</v>
       </c>
       <c r="Q4">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="R4" t="str">
         <v/>
@@ -706,55 +730,57 @@
         <v>JBB</v>
       </c>
       <c r="V4" t="str">
-        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama.</v>
-      </c>
-      <c r="W4" t="str">
-        <v>Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
-      </c>
-      <c r="X4" t="str">
-        <v>Optimalisasi transfer trip dan defense scheme antar GI.</v>
+        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA sedangkan IBT #4 Cilegon 500 MVA).</v>
+      </c>
+      <c r="W4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Ketidakseimbangan beban antara IBT Suralaya dan IBT Cilegon.
+2. Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
+      </c>
+      <c r="X4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW.
+2. Pemeliharaan IBT saat beban rendah dan Unit 3 beroperasi.</v>
       </c>
       <c r="Y4" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA.</v>
-      </c>
-    </row>
-    <row r="5">
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD Tahun 2026.</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="C5" t="str">
-        <v>Bay Evakuasi Unit 3 PLTU Suralaya</v>
+        <v>Bay IBT 4 Cilegon Baru (500/150 kV)</v>
       </c>
       <c r="D5" t="str">
-        <v>Bay Generator</v>
+        <v>Bay Interbus Transformer</v>
       </c>
       <c r="E5" t="str">
-        <v>Trafo Generator</v>
+        <v>ibt</v>
       </c>
       <c r="F5" t="str">
-        <v>Unit 3</v>
+        <v>Cilegon Baru</v>
       </c>
       <c r="G5" t="str">
-        <v>Pembangkit</v>
+        <v>busbar</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
       <c r="I5" t="str">
-        <v>SRLYA</v>
+        <v>CLBRU</v>
       </c>
       <c r="J5" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="K5">
         <v>1</v>
       </c>
       <c r="L5" t="str">
-        <v>500 kV</v>
+        <v>500/150 kV</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -766,16 +792,16 @@
         <v>Beroperasi</v>
       </c>
       <c r="P5" t="str">
-        <v>Normal</v>
+        <v>Sangat Rawan</v>
       </c>
       <c r="Q5">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="R5" t="str">
         <v/>
       </c>
       <c r="S5">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="T5" t="str">
         <v>Banten - Cilegon</v>
@@ -784,16 +810,17 @@
         <v>JBB</v>
       </c>
       <c r="V5" t="str">
-        <v>Evakuasi daya PLTU Suralaya Unit 3 (1. Pembangkit, 2. Trafo Step-Up, 3. CB).</v>
+        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #4 Cilegon 500 MVA sedangkan IBT #1,2 Suralaya 250 MVA).</v>
       </c>
       <c r="W5" t="str">
-        <v/>
+        <v>Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
       </c>
       <c r="X5" t="str">
-        <v/>
-      </c>
-      <c r="Y5" t="str">
-        <v/>
+        <v>Optimalisasi transfer trip dan defense scheme antar GI.</v>
+      </c>
+      <c r="Y5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jangka Pendek :
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. COD Tahun 2026.</v>
       </c>
     </row>
     <row r="6">
@@ -804,19 +831,19 @@
         <v/>
       </c>
       <c r="C6" t="str">
-        <v>Suralaya - Salira Indah (Sirkit 1)</v>
+        <v>SUTT 150 kV SRLYA - SLRDA</v>
       </c>
       <c r="D6" t="str">
-        <v>PHT</v>
+        <v>Saluran Udara (SUTT)</v>
       </c>
       <c r="E6" t="str">
-        <v>PHT</v>
+        <v>cb</v>
       </c>
       <c r="F6" t="str">
         <v>SRLYA</v>
       </c>
       <c r="G6" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -825,7 +852,7 @@
         <v>SLRDA</v>
       </c>
       <c r="J6" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="K6">
         <v>2</v>
@@ -834,7 +861,7 @@
         <v>150 kV</v>
       </c>
       <c r="M6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N6">
         <v>1</v>
@@ -846,13 +873,13 @@
         <v>Normal</v>
       </c>
       <c r="Q6">
-        <v>52</v>
-      </c>
-      <c r="R6">
-        <v>48</v>
+        <v>54</v>
+      </c>
+      <c r="R6" t="str">
+        <v/>
       </c>
       <c r="S6">
-        <v>12.5</v>
+        <v>14.2</v>
       </c>
       <c r="T6" t="str">
         <v>Banten - Cilegon</v>
@@ -881,28 +908,28 @@
         <v/>
       </c>
       <c r="C7" t="str">
-        <v>Suralaya - Salira Indah (Sirkit 2)</v>
+        <v>SUTT 150 kV SRLYA - PENDO</v>
       </c>
       <c r="D7" t="str">
-        <v>PHT</v>
+        <v>Saluran Udara (SUTT)</v>
       </c>
       <c r="E7" t="str">
-        <v>PHT</v>
+        <v>cb</v>
       </c>
       <c r="F7" t="str">
         <v>SRLYA</v>
       </c>
       <c r="G7" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7" t="str">
-        <v>SLRDA</v>
+        <v>PENDO</v>
       </c>
       <c r="J7" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="K7">
         <v>2</v>
@@ -911,10 +938,10 @@
         <v>150 kV</v>
       </c>
       <c r="M7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O7" t="str">
         <v>Beroperasi</v>
@@ -923,13 +950,13 @@
         <v>Normal</v>
       </c>
       <c r="Q7">
-        <v>52</v>
-      </c>
-      <c r="R7">
         <v>48</v>
       </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
       <c r="S7">
-        <v>12.5</v>
+        <v>12.8</v>
       </c>
       <c r="T7" t="str">
         <v>Banten - Cilegon</v>
@@ -958,19 +985,19 @@
         <v/>
       </c>
       <c r="C8" t="str">
-        <v>Salira Indah - Pendo</v>
+        <v>SUTT 150 kV Tie Line SLRDA - PENDO</v>
       </c>
       <c r="D8" t="str">
-        <v>PHT</v>
+        <v>Tie Line Interkoneksi</v>
       </c>
       <c r="E8" t="str">
-        <v>PHT</v>
+        <v>cb</v>
       </c>
       <c r="F8" t="str">
         <v>SLRDA</v>
       </c>
       <c r="G8" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H8">
         <v>2</v>
@@ -979,7 +1006,7 @@
         <v>PENDO</v>
       </c>
       <c r="J8" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="K8">
         <v>2</v>
@@ -1000,13 +1027,13 @@
         <v>Normal</v>
       </c>
       <c r="Q8">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="R8" t="str">
         <v/>
       </c>
       <c r="S8">
-        <v>8.4</v>
+        <v>6.4</v>
       </c>
       <c r="T8" t="str">
         <v>Banten - Cilegon</v>
@@ -1015,7 +1042,7 @@
         <v>JBB</v>
       </c>
       <c r="V8" t="str">
-        <v/>
+        <v>Interkoneksi antar bay busbar Salira Indah (SLRDA) dan Pendo (PENDO) di Tier 2.</v>
       </c>
       <c r="W8" t="str">
         <v/>
@@ -1027,7 +1054,7 @@
         <v/>
       </c>
     </row>
-    <row r="9">
+    <row r="9" xml:space="preserve">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1035,19 +1062,19 @@
         <v>3</v>
       </c>
       <c r="C9" t="str">
-        <v>Suralaya - Chandra Asri (PENI)</v>
+        <v>SUTT 150 kV SRLYA - PENI</v>
       </c>
       <c r="D9" t="str">
-        <v>PHT</v>
+        <v>Saluran Udara (SUTT)</v>
       </c>
       <c r="E9" t="str">
-        <v>PHT</v>
+        <v>cb</v>
       </c>
       <c r="F9" t="str">
         <v>SRLYA</v>
       </c>
       <c r="G9" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -1056,7 +1083,7 @@
         <v>PENI</v>
       </c>
       <c r="J9" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="K9">
         <v>2</v>
@@ -1077,13 +1104,13 @@
         <v>N-1</v>
       </c>
       <c r="Q9">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="R9" t="str">
         <v/>
       </c>
       <c r="S9">
-        <v>15.2</v>
+        <v>18.5</v>
       </c>
       <c r="T9" t="str">
         <v>Banten - Cilegon</v>
@@ -1092,19 +1119,22 @@
         <v>JBB</v>
       </c>
       <c r="V9" t="str">
-        <v>Ruas Penghantar Suralaya-PENI masih single phi.</v>
-      </c>
-      <c r="W9" t="str">
-        <v>Pemadaman apabila trip saat pemeliharaan KTT.</v>
-      </c>
-      <c r="X9" t="str">
-        <v>Penyesuaian jadwal pemeliharaan.</v>
-      </c>
-      <c r="Y9" t="str">
-        <v>Double phi COD 2030.</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>Ruas Penghantar Suralaya–MCCI–Cilegon dan Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
+      </c>
+      <c r="W9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Pemeliharaan Penghantar menjadi sulit dilakukan.
+2. Terjadi pemadaman apabila terdapat gangguan N–1–1.</v>
+      </c>
+      <c r="X9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Pemeliharaan Penghantar menyesuaikan jadwal dari KTT.
+2. Pengaturan konfigurasi jaringan saat pemeliharaan untuk mengurangi dampak padam.</v>
+      </c>
+      <c r="Y9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jangka Menengah :
+Usulan Double phi pada ruas Suralaya s.d Cilegon Lama (Kajian belum ada). Diusulkan COD Tahun 2030.</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1112,19 +1142,19 @@
         <v>3</v>
       </c>
       <c r="C10" t="str">
-        <v>Suralaya - MCCI</v>
+        <v>SUTT 150 kV SRLYA - MCCI5</v>
       </c>
       <c r="D10" t="str">
-        <v>PHT</v>
+        <v>Saluran Udara (SUTT)</v>
       </c>
       <c r="E10" t="str">
-        <v>PHT</v>
+        <v>cb</v>
       </c>
       <c r="F10" t="str">
         <v>SRLYA</v>
       </c>
       <c r="G10" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -1133,7 +1163,7 @@
         <v>MCCI5</v>
       </c>
       <c r="J10" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="K10">
         <v>2</v>
@@ -1154,13 +1184,13 @@
         <v>N-1</v>
       </c>
       <c r="Q10">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="R10" t="str">
         <v/>
       </c>
       <c r="S10">
-        <v>16.8</v>
+        <v>16.3</v>
       </c>
       <c r="T10" t="str">
         <v>Banten - Cilegon</v>
@@ -1169,57 +1199,60 @@
         <v>JBB</v>
       </c>
       <c r="V10" t="str">
-        <v>Ruas Penghantar Suralaya-MCCI-Cilegon masih single phi.</v>
-      </c>
-      <c r="W10" t="str">
-        <v>Pemadaman apabila terjadi trip.</v>
-      </c>
-      <c r="X10" t="str">
-        <v>Penyesuaian jadwal pemeliharaan dari KTT.</v>
-      </c>
-      <c r="Y10" t="str">
-        <v>Usulan double phi ruas Suralaya s.d Cilegon Lama.</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>Ruas Penghantar Suralaya–MCCI–Cilegon dan Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
+      </c>
+      <c r="W10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Pemeliharaan Penghantar menjadi sulit dilakukan.
+2. Terjadi pemadaman apabila terdapat gangguan N–1–1.</v>
+      </c>
+      <c r="X10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Pemeliharaan Penghantar menyesuaikan jadwal dari KTT.
+2. Pengaturan konfigurasi jaringan saat pemeliharaan.</v>
+      </c>
+      <c r="Y10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jangka Menengah :
+Usulan Double phi pada ruas Suralaya s.d Cilegon Lama. COD Tahun 2030.</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="C11" t="str">
-        <v>Cilegon Baru - Cilegon Lama (Sirkit 1)</v>
+        <v>SUTT 150 kV PENI - MTSUI</v>
       </c>
       <c r="D11" t="str">
-        <v>PHT</v>
+        <v>Saluran Udara (SUTT)</v>
       </c>
       <c r="E11" t="str">
-        <v>PHT</v>
+        <v>cb</v>
       </c>
       <c r="F11" t="str">
-        <v>CLBRU</v>
+        <v>PENI</v>
       </c>
       <c r="G11" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I11" t="str">
-        <v>CLGON</v>
+        <v>MTSUI</v>
       </c>
       <c r="J11" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="K11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L11" t="str">
         <v>150 kV</v>
       </c>
       <c r="M11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N11">
         <v>1</v>
@@ -1228,16 +1261,16 @@
         <v>Beroperasi</v>
       </c>
       <c r="P11" t="str">
-        <v>Normal</v>
+        <v>N-1</v>
       </c>
       <c r="Q11">
-        <v>54</v>
-      </c>
-      <c r="R11">
-        <v>50</v>
+        <v>68</v>
+      </c>
+      <c r="R11" t="str">
+        <v/>
       </c>
       <c r="S11">
-        <v>9.2</v>
+        <v>8.7</v>
       </c>
       <c r="T11" t="str">
         <v>Banten - Cilegon</v>
@@ -1246,16 +1279,18 @@
         <v>JBB</v>
       </c>
       <c r="V11" t="str">
-        <v/>
-      </c>
-      <c r="W11" t="str">
-        <v/>
+        <v>Ruas Penghantar Suralaya–MCCI–Cilegon dan Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
+      </c>
+      <c r="W11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Pemeliharaan Penghantar menjadi sulit dilakukan.
+2. Terjadi pemadaman apabila terdapat gangguan N–1–1.</v>
       </c>
       <c r="X11" t="str">
-        <v/>
-      </c>
-      <c r="Y11" t="str">
-        <v/>
+        <v>1. Pemeliharaan Penghantar menyesuaikan jadwal dari KTT.</v>
+      </c>
+      <c r="Y11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jangka Menengah :
+Usulan Double phi pada ruas Suralaya s.d Cilegon Lama. COD Tahun 2030.</v>
       </c>
     </row>
     <row r="12">
@@ -1263,31 +1298,31 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="C12" t="str">
-        <v>Cilegon Baru - Cilegon Lama (Sirkit 2)</v>
+        <v>SUTT 150 kV MCCI5 - CLGON</v>
       </c>
       <c r="D12" t="str">
-        <v>PHT</v>
+        <v>Saluran Udara (SUTT)</v>
       </c>
       <c r="E12" t="str">
-        <v>PHT</v>
+        <v>cb</v>
       </c>
       <c r="F12" t="str">
-        <v>CLBRU</v>
+        <v>MCCI5</v>
       </c>
       <c r="G12" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I12" t="str">
         <v>CLGON</v>
       </c>
       <c r="J12" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="K12">
         <v>2</v>
@@ -1296,25 +1331,25 @@
         <v>150 kV</v>
       </c>
       <c r="M12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O12" t="str">
         <v>Beroperasi</v>
       </c>
       <c r="P12" t="str">
-        <v>Normal</v>
+        <v>N-1</v>
       </c>
       <c r="Q12">
-        <v>54</v>
-      </c>
-      <c r="R12">
-        <v>50</v>
+        <v>65</v>
+      </c>
+      <c r="R12" t="str">
+        <v/>
       </c>
       <c r="S12">
-        <v>9.2</v>
+        <v>9.4</v>
       </c>
       <c r="T12" t="str">
         <v>Banten - Cilegon</v>
@@ -1323,16 +1358,16 @@
         <v>JBB</v>
       </c>
       <c r="V12" t="str">
-        <v/>
+        <v>Ruas Penghantar Suralaya–MCCI–Cilegon dan Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
       </c>
       <c r="W12" t="str">
-        <v/>
+        <v>Pemadaman apabila trip saat pemeliharaan KTT.</v>
       </c>
       <c r="X12" t="str">
-        <v/>
+        <v>Penyesuaian jadwal pemeliharaan dari KTT.</v>
       </c>
       <c r="Y12" t="str">
-        <v/>
+        <v>Usulan double phi ruas Suralaya s.d Cilegon Lama. COD Tahun 2030.</v>
       </c>
     </row>
     <row r="13">
@@ -1343,31 +1378,31 @@
         <v>3</v>
       </c>
       <c r="C13" t="str">
-        <v>Chandra Asri (PENI) - Mitsui (MTSUI)</v>
+        <v>SUTT 150 kV MTSUI - CLGON</v>
       </c>
       <c r="D13" t="str">
-        <v>PHT</v>
+        <v>Saluran Udara (SUTT)</v>
       </c>
       <c r="E13" t="str">
-        <v>PHT</v>
+        <v>cb</v>
       </c>
       <c r="F13" t="str">
-        <v>PENI</v>
+        <v>MTSUI</v>
       </c>
       <c r="G13" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H13">
+        <v>3</v>
+      </c>
+      <c r="I13" t="str">
+        <v>CLGON</v>
+      </c>
+      <c r="J13" t="str">
+        <v>busbar</v>
+      </c>
+      <c r="K13">
         <v>2</v>
-      </c>
-      <c r="I13" t="str">
-        <v>MTSUI</v>
-      </c>
-      <c r="J13" t="str">
-        <v>Busbar</v>
-      </c>
-      <c r="K13">
-        <v>3</v>
       </c>
       <c r="L13" t="str">
         <v>150 kV</v>
@@ -1385,13 +1420,13 @@
         <v>N-1</v>
       </c>
       <c r="Q13">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="R13" t="str">
         <v/>
       </c>
       <c r="S13">
-        <v>6.8</v>
+        <v>10.5</v>
       </c>
       <c r="T13" t="str">
         <v>Banten - Cilegon</v>
@@ -1400,16 +1435,16 @@
         <v>JBB</v>
       </c>
       <c r="V13" t="str">
-        <v>Ruas Peni-Mitsui-Cilegon masih single phi.</v>
+        <v>Ruas Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
       </c>
       <c r="W13" t="str">
-        <v>Pemadaman apabila trip.</v>
+        <v>Pemadaman apabila terjadi gangguan N-1.</v>
       </c>
       <c r="X13" t="str">
-        <v>Jadwal pemeliharaan KTT.</v>
+        <v>Pengaturan konfigurasi jaringan sistem Banten.</v>
       </c>
       <c r="Y13" t="str">
-        <v>Usulan double phi COD 2030.</v>
+        <v>Double phi ruas Suralaya s.d Cilegon Lama.</v>
       </c>
     </row>
     <row r="14">
@@ -1420,28 +1455,28 @@
         <v/>
       </c>
       <c r="C14" t="str">
-        <v>Mitsui (MTSUI) - Cilegon Lama</v>
+        <v>SUTT 150 kV CLBRU - CLGON Sirkit 1</v>
       </c>
       <c r="D14" t="str">
-        <v>PHT</v>
+        <v>Double Circuit Line 1</v>
       </c>
       <c r="E14" t="str">
-        <v>PHT</v>
+        <v>cb</v>
       </c>
       <c r="F14" t="str">
-        <v>MTSUI</v>
+        <v>CLBRU</v>
       </c>
       <c r="G14" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I14" t="str">
         <v>CLGON</v>
       </c>
       <c r="J14" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="K14">
         <v>2</v>
@@ -1450,7 +1485,7 @@
         <v>150 kV</v>
       </c>
       <c r="M14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N14">
         <v>1</v>
@@ -1462,13 +1497,13 @@
         <v>Normal</v>
       </c>
       <c r="Q14">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="R14" t="str">
         <v/>
       </c>
       <c r="S14">
-        <v>5.4</v>
+        <v>11.2</v>
       </c>
       <c r="T14" t="str">
         <v>Banten - Cilegon</v>
@@ -1477,7 +1512,7 @@
         <v>JBB</v>
       </c>
       <c r="V14" t="str">
-        <v/>
+        <v>Jalur ganda menghubungkan Cilegon Baru dan Cilegon Lama Sirkit 1.</v>
       </c>
       <c r="W14" t="str">
         <v/>
@@ -1497,40 +1532,40 @@
         <v/>
       </c>
       <c r="C15" t="str">
-        <v>Feeder Beban KTT SLFDO-1 (78 MVA)</v>
+        <v>SUTT 150 kV CLBRU - CLGON Sirkit 2</v>
       </c>
       <c r="D15" t="str">
-        <v>Feeder Beban</v>
+        <v>Double Circuit Line 2</v>
       </c>
       <c r="E15" t="str">
-        <v>Beban</v>
+        <v>cb</v>
       </c>
       <c r="F15" t="str">
-        <v>SLRDA</v>
+        <v>CLBRU</v>
       </c>
       <c r="G15" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15" t="str">
+        <v>CLGON</v>
+      </c>
+      <c r="J15" t="str">
+        <v>busbar</v>
+      </c>
+      <c r="K15">
         <v>2</v>
       </c>
-      <c r="I15" t="str">
-        <v>KTT SLFDO-1</v>
-      </c>
-      <c r="J15" t="str">
-        <v>Beban</v>
-      </c>
-      <c r="K15">
-        <v>3</v>
-      </c>
       <c r="L15" t="str">
-        <v>20 kV</v>
+        <v>150 kV</v>
       </c>
       <c r="M15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15" t="str">
         <v>Beroperasi</v>
@@ -1539,13 +1574,13 @@
         <v>Normal</v>
       </c>
       <c r="Q15">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="R15" t="str">
         <v/>
       </c>
       <c r="S15">
-        <v>1.2</v>
+        <v>11.2</v>
       </c>
       <c r="T15" t="str">
         <v>Banten - Cilegon</v>
@@ -1554,7 +1589,7 @@
         <v>JBB</v>
       </c>
       <c r="V15" t="str">
-        <v>Feeder Konsumen Industri KTT SLFDO-1</v>
+        <v>Jalur ganda menghubungkan Cilegon Baru dan Cilegon Lama Sirkit 2.</v>
       </c>
       <c r="W15" t="str">
         <v/>
@@ -1574,34 +1609,34 @@
         <v/>
       </c>
       <c r="C16" t="str">
-        <v>Feeder Beban KTT SLFDO-2 (30 MVA)</v>
+        <v>Bay Trafo Distribusi SRLYA</v>
       </c>
       <c r="D16" t="str">
-        <v>Feeder Beban</v>
+        <v>Bay Trafo</v>
       </c>
       <c r="E16" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="F16" t="str">
-        <v>SLRDA</v>
+        <v>SRLYA</v>
       </c>
       <c r="G16" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Trafo Distribusi SRLYA</v>
+      </c>
+      <c r="J16" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="K16">
         <v>2</v>
       </c>
-      <c r="I16" t="str">
-        <v>KTT SLFDO-2</v>
-      </c>
-      <c r="J16" t="str">
-        <v>Beban</v>
-      </c>
-      <c r="K16">
-        <v>3</v>
-      </c>
       <c r="L16" t="str">
-        <v>20 kV</v>
+        <v>150/20 kV</v>
       </c>
       <c r="M16">
         <v>1</v>
@@ -1616,13 +1651,13 @@
         <v>Normal</v>
       </c>
       <c r="Q16">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="R16" t="str">
         <v/>
       </c>
       <c r="S16">
-        <v>1.2</v>
+        <v>0.1</v>
       </c>
       <c r="T16" t="str">
         <v>Banten - Cilegon</v>
@@ -1631,7 +1666,7 @@
         <v>JBB</v>
       </c>
       <c r="V16" t="str">
-        <v>Feeder Konsumen Industri KTT SLFDO-2</v>
+        <v>Trafo pemakaian sendiri / distribusi lokal 150/20 kV Suralaya.</v>
       </c>
       <c r="W16" t="str">
         <v/>
@@ -1651,34 +1686,34 @@
         <v/>
       </c>
       <c r="C17" t="str">
-        <v>Feeder Beban KTT PENDO (35 MVA)</v>
+        <v>Bay Trafo Distribusi CLBRU</v>
       </c>
       <c r="D17" t="str">
-        <v>Feeder Beban</v>
+        <v>Bay Trafo</v>
       </c>
       <c r="E17" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="F17" t="str">
-        <v>PENDO</v>
+        <v>CLBRU</v>
       </c>
       <c r="G17" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Trafo Distribusi CLBRU</v>
+      </c>
+      <c r="J17" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="K17">
         <v>2</v>
       </c>
-      <c r="I17" t="str">
-        <v>KTT PENDO</v>
-      </c>
-      <c r="J17" t="str">
-        <v>Beban</v>
-      </c>
-      <c r="K17">
-        <v>3</v>
-      </c>
       <c r="L17" t="str">
-        <v>20 kV</v>
+        <v>150/20 kV</v>
       </c>
       <c r="M17">
         <v>1</v>
@@ -1693,13 +1728,13 @@
         <v>Normal</v>
       </c>
       <c r="Q17">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="R17" t="str">
         <v/>
       </c>
       <c r="S17">
-        <v>0.8</v>
+        <v>0.1</v>
       </c>
       <c r="T17" t="str">
         <v>Banten - Cilegon</v>
@@ -1708,7 +1743,7 @@
         <v>JBB</v>
       </c>
       <c r="V17" t="str">
-        <v>Feeder Konsumen Industri KTT PENDO</v>
+        <v>Trafo distribusi lokal 150/20 kV Cilegon Baru.</v>
       </c>
       <c r="W17" t="str">
         <v/>
@@ -1725,37 +1760,37 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="C18" t="str">
-        <v>Feeder Beban KTT PENI (40 MVA)</v>
+        <v>Feeder Trafo SLRDA ke KTT SLFDO-1</v>
       </c>
       <c r="D18" t="str">
-        <v>Feeder Beban</v>
+        <v>Feeder KTT</v>
       </c>
       <c r="E18" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="F18" t="str">
-        <v>PENI</v>
+        <v>SLRDA</v>
       </c>
       <c r="G18" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H18">
         <v>2</v>
       </c>
       <c r="I18" t="str">
-        <v>KTT PENI</v>
+        <v>KTT SLFDO-1</v>
       </c>
       <c r="J18" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="K18">
         <v>3</v>
       </c>
       <c r="L18" t="str">
-        <v>20 kV</v>
+        <v>150/20 kV</v>
       </c>
       <c r="M18">
         <v>1</v>
@@ -1767,16 +1802,16 @@
         <v>Beroperasi</v>
       </c>
       <c r="P18" t="str">
-        <v>N-1</v>
+        <v>Normal</v>
       </c>
       <c r="Q18">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="R18" t="str">
         <v/>
       </c>
       <c r="S18">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="T18" t="str">
         <v>Banten - Cilegon</v>
@@ -1785,7 +1820,7 @@
         <v>JBB</v>
       </c>
       <c r="V18" t="str">
-        <v>Feeder Konsumen Industri KTT PENI</v>
+        <v>Suplai konsumen KTT SLFDO-1 Kapasitas 78 MVA</v>
       </c>
       <c r="W18" t="str">
         <v/>
@@ -1805,37 +1840,37 @@
         <v/>
       </c>
       <c r="C19" t="str">
-        <v>Feeder Beban KTT LCI (115 MVA)</v>
+        <v>Feeder Trafo SLRDA ke KTT SLFDO-2</v>
       </c>
       <c r="D19" t="str">
-        <v>Feeder Beban</v>
+        <v>Feeder KTT</v>
       </c>
       <c r="E19" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="F19" t="str">
-        <v>PENI</v>
+        <v>SLRDA</v>
       </c>
       <c r="G19" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H19">
         <v>2</v>
       </c>
       <c r="I19" t="str">
-        <v>KTT LCI</v>
+        <v>KTT SLFDO-2</v>
       </c>
       <c r="J19" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="K19">
         <v>3</v>
       </c>
       <c r="L19" t="str">
-        <v>20 kV</v>
+        <v>150/20 kV</v>
       </c>
       <c r="M19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N19">
         <v>1</v>
@@ -1847,13 +1882,13 @@
         <v>Normal</v>
       </c>
       <c r="Q19">
-        <v>58</v>
-      </c>
-      <c r="R19">
-        <v>57</v>
+        <v>65</v>
+      </c>
+      <c r="R19" t="str">
+        <v/>
       </c>
       <c r="S19">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="T19" t="str">
         <v>Banten - Cilegon</v>
@@ -1862,7 +1897,7 @@
         <v>JBB</v>
       </c>
       <c r="V19" t="str">
-        <v>Feeder Konsumen Industri KTT LCI</v>
+        <v>Suplai konsumen KTT SLFDO-2 Kapasitas 30 MVA</v>
       </c>
       <c r="W19" t="str">
         <v/>
@@ -1882,34 +1917,34 @@
         <v/>
       </c>
       <c r="C20" t="str">
-        <v>Feeder Beban KTT MCCI (40 MVA)</v>
+        <v>Feeder Trafo PENDO ke KTT PENDO</v>
       </c>
       <c r="D20" t="str">
-        <v>Feeder Beban</v>
+        <v>Feeder KTT</v>
       </c>
       <c r="E20" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="F20" t="str">
-        <v>MCCI5</v>
+        <v>PENDO</v>
       </c>
       <c r="G20" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H20">
         <v>2</v>
       </c>
       <c r="I20" t="str">
-        <v>KTT MCCI</v>
+        <v>KTT PENDO</v>
       </c>
       <c r="J20" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="K20">
         <v>3</v>
       </c>
       <c r="L20" t="str">
-        <v>20 kV</v>
+        <v>150/20 kV</v>
       </c>
       <c r="M20">
         <v>1</v>
@@ -1924,13 +1959,13 @@
         <v>Normal</v>
       </c>
       <c r="Q20">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="R20" t="str">
         <v/>
       </c>
       <c r="S20">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="T20" t="str">
         <v>Banten - Cilegon</v>
@@ -1939,7 +1974,7 @@
         <v>JBB</v>
       </c>
       <c r="V20" t="str">
-        <v>Feeder Konsumen Industri KTT MCCI</v>
+        <v>Suplai konsumen KTT PENDO Kapasitas 35 MVA</v>
       </c>
       <c r="W20" t="str">
         <v/>
@@ -1956,37 +1991,37 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="C21" t="str">
-        <v>Feeder Beban KTT MTSUI (31 MVA)</v>
+        <v>Feeder Trafo PENI ke KTT PENI</v>
       </c>
       <c r="D21" t="str">
-        <v>Feeder Beban</v>
+        <v>Feeder KTT</v>
       </c>
       <c r="E21" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="F21" t="str">
-        <v>MTSUI</v>
+        <v>PENI</v>
       </c>
       <c r="G21" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="H21">
+        <v>2</v>
+      </c>
+      <c r="I21" t="str">
+        <v>KTT PENI</v>
+      </c>
+      <c r="J21" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="K21">
         <v>3</v>
       </c>
-      <c r="I21" t="str">
-        <v>KTT MTSUI</v>
-      </c>
-      <c r="J21" t="str">
-        <v>Beban</v>
-      </c>
-      <c r="K21">
-        <v>4</v>
-      </c>
       <c r="L21" t="str">
-        <v>20 kV</v>
+        <v>150/20 kV</v>
       </c>
       <c r="M21">
         <v>1</v>
@@ -1998,16 +2033,16 @@
         <v>Beroperasi</v>
       </c>
       <c r="P21" t="str">
-        <v>Normal</v>
+        <v>N-1</v>
       </c>
       <c r="Q21">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="R21" t="str">
         <v/>
       </c>
       <c r="S21">
-        <v>0.4</v>
+        <v>1.1</v>
       </c>
       <c r="T21" t="str">
         <v>Banten - Cilegon</v>
@@ -2016,28 +2051,586 @@
         <v>JBB</v>
       </c>
       <c r="V21" t="str">
-        <v>Feeder Konsumen Industri KTT Mitsui</v>
+        <v>Suplai konsumen KTT PENI Chandra Asri Kapasitas 40 MVA</v>
       </c>
       <c r="W21" t="str">
-        <v/>
+        <v>Terdapat risiko suplai saat pemeliharaan ruas single phi.</v>
       </c>
       <c r="X21" t="str">
-        <v/>
+        <v>Penyesuaian jadwal dengan konsumen industri.</v>
       </c>
       <c r="Y21" t="str">
+        <v>Usulan double phi transmisi 150 kV.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22" t="str">
+        <v>Feeder Trafo PENI ke KTT LCI</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Feeder KTT</v>
+      </c>
+      <c r="E22" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PENI</v>
+      </c>
+      <c r="G22" t="str">
+        <v>busbar</v>
+      </c>
+      <c r="H22">
+        <v>2</v>
+      </c>
+      <c r="I22" t="str">
+        <v>KTT LCI</v>
+      </c>
+      <c r="J22" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="K22">
+        <v>3</v>
+      </c>
+      <c r="L22" t="str">
+        <v>150/20 kV</v>
+      </c>
+      <c r="M22">
+        <v>2</v>
+      </c>
+      <c r="N22">
+        <v>1</v>
+      </c>
+      <c r="O22" t="str">
+        <v>Beroperasi</v>
+      </c>
+      <c r="P22" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q22">
+        <v>64</v>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
+      <c r="S22">
+        <v>1.5</v>
+      </c>
+      <c r="T22" t="str">
+        <v>Banten - Cilegon</v>
+      </c>
+      <c r="U22" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V22" t="str">
+        <v>Suplai 2 sirkit konsumen KTT LCI Kapasitas 115 MVA</v>
+      </c>
+      <c r="W22" t="str">
+        <v/>
+      </c>
+      <c r="X22" t="str">
+        <v/>
+      </c>
+      <c r="Y22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
+        <v>Feeder Trafo MCCI5 ke KTT MCCI</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Feeder KTT</v>
+      </c>
+      <c r="E23" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="F23" t="str">
+        <v>MCCI5</v>
+      </c>
+      <c r="G23" t="str">
+        <v>busbar</v>
+      </c>
+      <c r="H23">
+        <v>2</v>
+      </c>
+      <c r="I23" t="str">
+        <v>KTT MCCI</v>
+      </c>
+      <c r="J23" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="K23">
+        <v>3</v>
+      </c>
+      <c r="L23" t="str">
+        <v>150/20 kV</v>
+      </c>
+      <c r="M23">
+        <v>1</v>
+      </c>
+      <c r="N23">
+        <v>1</v>
+      </c>
+      <c r="O23" t="str">
+        <v>Beroperasi</v>
+      </c>
+      <c r="P23" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q23">
+        <v>55</v>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23">
+        <v>0.9</v>
+      </c>
+      <c r="T23" t="str">
+        <v>Banten - Cilegon</v>
+      </c>
+      <c r="U23" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V23" t="str">
+        <v>Suplai konsumen KTT MCCI Kapasitas 40 MVA</v>
+      </c>
+      <c r="W23" t="str">
+        <v/>
+      </c>
+      <c r="X23" t="str">
+        <v/>
+      </c>
+      <c r="Y23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v>Bay Trafo Distribusi CLGON</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Bay Trafo</v>
+      </c>
+      <c r="E24" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="F24" t="str">
+        <v>CLGON</v>
+      </c>
+      <c r="G24" t="str">
+        <v>busbar</v>
+      </c>
+      <c r="H24">
+        <v>2</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Trafo Distribusi CLGON</v>
+      </c>
+      <c r="J24" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="K24">
+        <v>3</v>
+      </c>
+      <c r="L24" t="str">
+        <v>150/20 kV</v>
+      </c>
+      <c r="M24">
+        <v>1</v>
+      </c>
+      <c r="N24">
+        <v>1</v>
+      </c>
+      <c r="O24" t="str">
+        <v>Beroperasi</v>
+      </c>
+      <c r="P24" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q24">
+        <v>52</v>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24">
+        <v>0.1</v>
+      </c>
+      <c r="T24" t="str">
+        <v>Banten - Cilegon</v>
+      </c>
+      <c r="U24" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V24" t="str">
+        <v>Trafo distribusi lokal 150/20 kV Cilegon Lama.</v>
+      </c>
+      <c r="W24" t="str">
+        <v/>
+      </c>
+      <c r="X24" t="str">
+        <v/>
+      </c>
+      <c r="Y24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v/>
+      </c>
+      <c r="C25" t="str">
+        <v>Feeder Trafo MTSUI ke KTT MTSUI</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Feeder KTT</v>
+      </c>
+      <c r="E25" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="F25" t="str">
+        <v>MTSUI</v>
+      </c>
+      <c r="G25" t="str">
+        <v>busbar</v>
+      </c>
+      <c r="H25">
+        <v>3</v>
+      </c>
+      <c r="I25" t="str">
+        <v>KTT MTSUI</v>
+      </c>
+      <c r="J25" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="K25">
+        <v>4</v>
+      </c>
+      <c r="L25" t="str">
+        <v>150/20 kV</v>
+      </c>
+      <c r="M25">
+        <v>1</v>
+      </c>
+      <c r="N25">
+        <v>1</v>
+      </c>
+      <c r="O25" t="str">
+        <v>Beroperasi</v>
+      </c>
+      <c r="P25" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q25">
+        <v>50</v>
+      </c>
+      <c r="R25" t="str">
+        <v/>
+      </c>
+      <c r="S25">
+        <v>0.7</v>
+      </c>
+      <c r="T25" t="str">
+        <v>Banten - Cilegon</v>
+      </c>
+      <c r="U25" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V25" t="str">
+        <v>Suplai konsumen KTT MTSUI Kapasitas 31 MVA</v>
+      </c>
+      <c r="W25" t="str">
+        <v/>
+      </c>
+      <c r="X25" t="str">
+        <v/>
+      </c>
+      <c r="Y25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v>Bay Feeder CLBRU ke KSTEL (Rencana)</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Bay Rencana</v>
+      </c>
+      <c r="E26" t="str">
+        <v>cb</v>
+      </c>
+      <c r="F26" t="str">
+        <v>CLBRU</v>
+      </c>
+      <c r="G26" t="str">
+        <v>busbar</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26" t="str">
+        <v>KSTEL</v>
+      </c>
+      <c r="J26" t="str">
+        <v>cb</v>
+      </c>
+      <c r="K26">
+        <v>3</v>
+      </c>
+      <c r="L26" t="str">
+        <v>150 kV</v>
+      </c>
+      <c r="M26">
+        <v>1</v>
+      </c>
+      <c r="N26">
+        <v>1</v>
+      </c>
+      <c r="O26" t="str">
+        <v>Rencana</v>
+      </c>
+      <c r="P26" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q26">
+        <v>0</v>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
+      <c r="S26">
+        <v>3.5</v>
+      </c>
+      <c r="T26" t="str">
+        <v>Banten - Cilegon</v>
+      </c>
+      <c r="U26" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V26" t="str">
+        <v>Bay Rencana Penghantar KSTEL (Dashed Line)</v>
+      </c>
+      <c r="W26" t="str">
+        <v/>
+      </c>
+      <c r="X26" t="str">
+        <v/>
+      </c>
+      <c r="Y26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v>Bay Feeder CLBRU ke POSCO (Rencana)</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Bay Rencana</v>
+      </c>
+      <c r="E27" t="str">
+        <v>cb</v>
+      </c>
+      <c r="F27" t="str">
+        <v>CLBRU</v>
+      </c>
+      <c r="G27" t="str">
+        <v>busbar</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27" t="str">
+        <v>POSCO</v>
+      </c>
+      <c r="J27" t="str">
+        <v>cb</v>
+      </c>
+      <c r="K27">
+        <v>3</v>
+      </c>
+      <c r="L27" t="str">
+        <v>150 kV</v>
+      </c>
+      <c r="M27">
+        <v>1</v>
+      </c>
+      <c r="N27">
+        <v>1</v>
+      </c>
+      <c r="O27" t="str">
+        <v>Rencana</v>
+      </c>
+      <c r="P27" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q27">
+        <v>0</v>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27">
+        <v>4.2</v>
+      </c>
+      <c r="T27" t="str">
+        <v>Banten - Cilegon</v>
+      </c>
+      <c r="U27" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V27" t="str">
+        <v>Bay Rencana Penghantar POSCO (Dashed Line)</v>
+      </c>
+      <c r="W27" t="str">
+        <v/>
+      </c>
+      <c r="X27" t="str">
+        <v/>
+      </c>
+      <c r="Y27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v>Bay Feeder CLGON ke KSTEL (Rencana)</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Bay Rencana</v>
+      </c>
+      <c r="E28" t="str">
+        <v>cb</v>
+      </c>
+      <c r="F28" t="str">
+        <v>CLGON</v>
+      </c>
+      <c r="G28" t="str">
+        <v>busbar</v>
+      </c>
+      <c r="H28">
+        <v>2</v>
+      </c>
+      <c r="I28" t="str">
+        <v>KSTEL</v>
+      </c>
+      <c r="J28" t="str">
+        <v>cb</v>
+      </c>
+      <c r="K28">
+        <v>3</v>
+      </c>
+      <c r="L28" t="str">
+        <v>150 kV</v>
+      </c>
+      <c r="M28">
+        <v>1</v>
+      </c>
+      <c r="N28">
+        <v>1</v>
+      </c>
+      <c r="O28" t="str">
+        <v>Rencana</v>
+      </c>
+      <c r="P28" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="Q28">
+        <v>0</v>
+      </c>
+      <c r="R28" t="str">
+        <v/>
+      </c>
+      <c r="S28">
+        <v>2.8</v>
+      </c>
+      <c r="T28" t="str">
+        <v>Banten - Cilegon</v>
+      </c>
+      <c r="U28" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="V28" t="str">
+        <v>Bay Rencana Penghantar KSTEL dari CLGON (Dashed Line)</v>
+      </c>
+      <c r="W28" t="str">
+        <v/>
+      </c>
+      <c r="X28" t="str">
+        <v/>
+      </c>
+      <c r="Y28" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Y21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y28"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q28"/>
+  <cols>
+    <col min="1" max="1" width="5.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" customWidth="1"/>
+    <col min="14" max="14" width="45.83203125" customWidth="1"/>
+    <col min="15" max="15" width="35.83203125" customWidth="1"/>
+    <col min="16" max="16" width="35.83203125" customWidth="1"/>
+    <col min="17" max="17" width="35.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2103,10 +2696,10 @@
         <v>Suralaya Baru</v>
       </c>
       <c r="D2" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="E2" t="str">
-        <v>Normal</v>
+        <v>Panjang (Wide Busbar)</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -2133,7 +2726,7 @@
         <v>JBB</v>
       </c>
       <c r="N2" t="str">
-        <v>Busbar 500 kV Suralaya Baru</v>
+        <v>Rel Busbar 500 kV Suralaya Baru (Warna Biru)</v>
       </c>
       <c r="O2" t="str">
         <v/>
@@ -2156,10 +2749,10 @@
         <v>Suralaya</v>
       </c>
       <c r="D3" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="E3" t="str">
-        <v>Normal</v>
+        <v>Panjang (Wide Busbar)</v>
       </c>
       <c r="F3" t="str">
         <v/>
@@ -2186,7 +2779,7 @@
         <v>JBB</v>
       </c>
       <c r="N3" t="str">
-        <v>Busbar 500 kV Suralaya</v>
+        <v>Rel Busbar 500 kV Suralaya (Warna Biru)</v>
       </c>
       <c r="O3" t="str">
         <v/>
@@ -2209,10 +2802,10 @@
         <v>Cilegon Baru</v>
       </c>
       <c r="D4" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="E4" t="str">
-        <v>Normal</v>
+        <v>Panjang (Wide Busbar)</v>
       </c>
       <c r="F4" t="str">
         <v/>
@@ -2239,7 +2832,7 @@
         <v>JBB</v>
       </c>
       <c r="N4" t="str">
-        <v>Busbar 500 kV Cilegon Baru</v>
+        <v>Rel Busbar 500 kV Cilegon Baru (Warna Biru)</v>
       </c>
       <c r="O4" t="str">
         <v/>
@@ -2262,7 +2855,7 @@
         <v>Unit 3</v>
       </c>
       <c r="D5" t="str">
-        <v>Pembangkit</v>
+        <v>generator</v>
       </c>
       <c r="E5" t="str">
         <v>Normal</v>
@@ -2292,7 +2885,7 @@
         <v>JBB</v>
       </c>
       <c r="N5" t="str">
-        <v>Bay Pembangkit: 1. Pembangkit, 2. Trafo Generator, 3. CB</v>
+        <v>Generator Pembangkit Unit 3 (Lingkaran Hijau + Simbol AC ~) dengan Step-up GSUT</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -2304,7 +2897,7 @@
         <v/>
       </c>
     </row>
-    <row r="6">
+    <row r="6" xml:space="preserve">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2315,7 +2908,7 @@
         <v>IBT 2 SRL-BARU</v>
       </c>
       <c r="D6" t="str">
-        <v>IBT</v>
+        <v>ibt</v>
       </c>
       <c r="E6" t="str">
         <v>Normal</v>
@@ -2345,19 +2938,24 @@
         <v>JBB</v>
       </c>
       <c r="N6" t="str">
-        <v>Pembebanan IBT–1,2 Suralaya tidak memenuhi kriteria N–1 saat PLTU Suralaya unit–3 tidak beroperasi.</v>
-      </c>
-      <c r="O6" t="str">
-        <v>Pemadaman apabila trip salah satu IBT.</v>
-      </c>
-      <c r="P6" t="str">
-        <v>Terpasang DS OLS IBT 1,2 Suralaya.</v>
-      </c>
-      <c r="Q6" t="str">
-        <v>Uprating IBT–1 &amp; 2 dari 250 MVA menjadi 500 MVA.</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>Pembebanan IBT–1,2 Suralaya tidak memenuhi kriteria N–1 saat PLTU Suralaya unit–3 tidak beroperasi dan IBT–4 Cilegon masuk sub sistem Cilegon.</v>
+      </c>
+      <c r="O6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Pemeliharaan IBT sulit dilakukan.
+2. Pertumbuhan beban menjadi terhambat.
+3. Terjadi pemadaman apabila trip salah satu IBT di Suralaya.</v>
+      </c>
+      <c r="P6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW.
+2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan target total 137 MW.
+3. Pemeliharaan IBT saat beban rendah.</v>
+      </c>
+      <c r="Q6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jangka Pendek :
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. COD Tahun 2025.</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2368,7 +2966,7 @@
         <v>IBT 1 SRLYA</v>
       </c>
       <c r="D7" t="str">
-        <v>IBT</v>
+        <v>ibt</v>
       </c>
       <c r="E7" t="str">
         <v>Normal</v>
@@ -2398,19 +2996,22 @@
         <v>JBB</v>
       </c>
       <c r="N7" t="str">
-        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA).</v>
-      </c>
-      <c r="O7" t="str">
-        <v>Overload pada IBT Suralaya.</v>
-      </c>
-      <c r="P7" t="str">
-        <v>Terpasang DS OLS IBT 1,2 Suralaya.</v>
-      </c>
-      <c r="Q7" t="str">
-        <v>Uprating IBT–1 &amp; 2 dari 250 MVA menjadi 500 MVA.</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA sedangkan IBT #4 Cilegon 500 MVA).</v>
+      </c>
+      <c r="O7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Ketidakseimbangan beban antara IBT Suralaya dan IBT Cilegon.
+2. Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
+      </c>
+      <c r="P7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya.
+2. Pemeliharaan IBT saat beban rendah.</v>
+      </c>
+      <c r="Q7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jangka Pendek :
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. COD Tahun 2026.</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2421,7 +3022,7 @@
         <v>IBT 4 CLBRU</v>
       </c>
       <c r="D8" t="str">
-        <v>IBT</v>
+        <v>ibt</v>
       </c>
       <c r="E8" t="str">
         <v>Normal</v>
@@ -2454,13 +3055,14 @@
         <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #4 Cilegon 500 MVA).</v>
       </c>
       <c r="O8" t="str">
-        <v>Ketidakseimbangan beban.</v>
+        <v>Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
       </c>
       <c r="P8" t="str">
-        <v>Optimalisasi transfer trip antar GI.</v>
-      </c>
-      <c r="Q8" t="str">
-        <v>Uprating IBT–1 &amp; 2 Suralaya menjadi 500 MVA.</v>
+        <v>Optimalisasi transfer trip dan defense scheme antar GI.</v>
+      </c>
+      <c r="Q8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jangka Pendek :
+Uprating IBT–1 &amp; 2 Suralaya menjadi 500 MVA.</v>
       </c>
     </row>
     <row r="9">
@@ -2468,13 +3070,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>GI Suralaya 150 kV (Rel Busbar)</v>
+        <v>Gardu Induk SRLYA (150 kV)</v>
       </c>
       <c r="C9" t="str">
         <v>SRLYA</v>
       </c>
       <c r="D9" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="E9" t="str">
         <v>Panjang (Wide Busbar)</v>
@@ -2504,7 +3106,7 @@
         <v>JBB</v>
       </c>
       <c r="N9" t="str">
-        <v>Busbar 150 kV Suralaya (Menghubungkan IBT 1, IBT 2, dan Saluran Distribusi)</v>
+        <v>Busbar Utama 150 kV Suralaya (Tier 1, Merah Panjang menampung Unit 3, IBT 1, IBT 2, dan 5 Saluran ke Bawah)</v>
       </c>
       <c r="O9" t="str">
         <v/>
@@ -2521,13 +3123,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>GI Cilegon Baru 150 kV (Rel Busbar)</v>
+        <v>Gardu Induk CLBRU (150 kV)</v>
       </c>
       <c r="C10" t="str">
         <v>CLBRU</v>
       </c>
       <c r="D10" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="E10" t="str">
         <v>Panjang (Wide Busbar)</v>
@@ -2557,7 +3159,7 @@
         <v>JBB</v>
       </c>
       <c r="N10" t="str">
-        <v>Busbar 150 kV Cilegon Baru</v>
+        <v>Busbar Utama 150 kV Cilegon Baru (Tier 1, Merah Panjang menghubungkan IBT 4 ke CLGON, Trafo Lokal, KSTEL, POSCO)</v>
       </c>
       <c r="O10" t="str">
         <v/>
@@ -2574,13 +3176,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>GI Salira Indah</v>
+        <v>Gardu Induk SLRDA (150 kV)</v>
       </c>
       <c r="C11" t="str">
         <v>SLRDA</v>
       </c>
       <c r="D11" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="E11" t="str">
         <v>Normal</v>
@@ -2610,7 +3212,7 @@
         <v>JBB</v>
       </c>
       <c r="N11" t="str">
-        <v>Gardu Induk Salira Indah</v>
+        <v>Gardu Induk Salira Indah (Tier 2, Menyuplai KTT SLFDO-1 &amp; SLFDO-2)</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -2627,13 +3229,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>GI Pendo</v>
+        <v>Gardu Induk PENDO (150 kV)</v>
       </c>
       <c r="C12" t="str">
         <v>PENDO</v>
       </c>
       <c r="D12" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="E12" t="str">
         <v>Normal</v>
@@ -2663,7 +3265,7 @@
         <v>JBB</v>
       </c>
       <c r="N12" t="str">
-        <v>Gardu Induk Pendo</v>
+        <v>Gardu Induk Pendo (Tier 2, Menyuplai KTT PENDO 35 MVA)</v>
       </c>
       <c r="O12" t="str">
         <v/>
@@ -2680,13 +3282,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>GI Chandra Asri (PENI)</v>
+        <v>Gardu Induk PENI (150 kV)</v>
       </c>
       <c r="C13" t="str">
         <v>PENI</v>
       </c>
       <c r="D13" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="E13" t="str">
         <v>Normal</v>
@@ -2716,16 +3318,16 @@
         <v>JBB</v>
       </c>
       <c r="N13" t="str">
-        <v>Ruas Penghantar Suralaya-PENI masih single phi.</v>
+        <v>Ruas Penghantar Suralaya–PENI–Mitsui–Cilegon masih single phi.</v>
       </c>
       <c r="O13" t="str">
-        <v>Pemadaman apabila terdapat gangguan N-1-1.</v>
+        <v>Pemadaman apabila terdapat gangguan N–1–1.</v>
       </c>
       <c r="P13" t="str">
-        <v>Pemeliharaan mengikuti jadwal KTT.</v>
+        <v>Pemeliharaan mengikuti jadwal KTT industri.</v>
       </c>
       <c r="Q13" t="str">
-        <v>Double phi COD 2030.</v>
+        <v>Double phi transmisi 150 kV COD 2030.</v>
       </c>
     </row>
     <row r="14">
@@ -2733,13 +3335,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>GI Mitsubishi Chemical (MCCI)</v>
+        <v>Gardu Induk MCCI5 (150 kV)</v>
       </c>
       <c r="C14" t="str">
         <v>MCCI5</v>
       </c>
       <c r="D14" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="E14" t="str">
         <v>Normal</v>
@@ -2769,13 +3371,13 @@
         <v>JBB</v>
       </c>
       <c r="N14" t="str">
-        <v>Ruas Penghantar Suralaya-MCCI-Cilegon masih single phi.</v>
+        <v>Ruas Penghantar Suralaya–MCCI–Cilegon masih single phi.</v>
       </c>
       <c r="O14" t="str">
-        <v>Pemadaman apabila gangguan.</v>
+        <v>Pemadaman apabila trip saat pemeliharaan KTT.</v>
       </c>
       <c r="P14" t="str">
-        <v>Penyesuaian jadwal pemeliharaan.</v>
+        <v>Penyesuaian jadwal pemeliharaan dari KTT.</v>
       </c>
       <c r="Q14" t="str">
         <v>Usulan double phi ruas Suralaya s.d Cilegon Lama.</v>
@@ -2786,13 +3388,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>GI Cilegon Lama</v>
+        <v>Gardu Induk CLGON (150 kV)</v>
       </c>
       <c r="C15" t="str">
         <v>CLGON</v>
       </c>
       <c r="D15" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="E15" t="str">
         <v>Normal</v>
@@ -2822,7 +3424,7 @@
         <v>JBB</v>
       </c>
       <c r="N15" t="str">
-        <v>Gardu Induk Cilegon Lama</v>
+        <v>Gardu Induk Cilegon Lama (Menerima double circuit dari CLBRU, serta loop dari MCCI5 dan MTSUI)</v>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -2839,13 +3441,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>GI Mitsui (MTSUI)</v>
+        <v>Gardu Induk MTSUI (150 kV)</v>
       </c>
       <c r="C16" t="str">
         <v>MTSUI</v>
       </c>
       <c r="D16" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="E16" t="str">
         <v>Normal</v>
@@ -2875,16 +3477,16 @@
         <v>JBB</v>
       </c>
       <c r="N16" t="str">
-        <v>Ruas Mitsui-Cilegon single phi</v>
+        <v>Ruas Peni–Mitsui–Cilegon masih single phi (Tier 3).</v>
       </c>
       <c r="O16" t="str">
-        <v/>
+        <v>Terjadi pemadaman apabila trip N-1.</v>
       </c>
       <c r="P16" t="str">
-        <v/>
+        <v>Pengaturan konfigurasi jaringan.</v>
       </c>
       <c r="Q16" t="str">
-        <v/>
+        <v>Double phi ruas Suralaya s.d Cilegon Lama.</v>
       </c>
     </row>
     <row r="17">
@@ -2892,13 +3494,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>Konsumen KTT SLFDO-1 (78 MVA)</v>
+        <v>KTT SLFDO-1</v>
       </c>
       <c r="C17" t="str">
         <v>KTT SLFDO-1</v>
       </c>
       <c r="D17" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="E17" t="str">
         <v>Normal</v>
@@ -2928,7 +3530,7 @@
         <v>JBB</v>
       </c>
       <c r="N17" t="str">
-        <v>Konsumen Tegangan Tinggi SLFDO-1</v>
+        <v>Konsumen Tegangan Tinggi SLFDO-1 (78 MVA)</v>
       </c>
       <c r="O17" t="str">
         <v/>
@@ -2945,13 +3547,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>Konsumen KTT SLFDO-2 (30 MVA)</v>
+        <v>KTT SLFDO-2</v>
       </c>
       <c r="C18" t="str">
         <v>KTT SLFDO-2</v>
       </c>
       <c r="D18" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="E18" t="str">
         <v>Normal</v>
@@ -2981,7 +3583,7 @@
         <v>JBB</v>
       </c>
       <c r="N18" t="str">
-        <v>Konsumen Tegangan Tinggi SLFDO-2</v>
+        <v>Konsumen Tegangan Tinggi SLFDO-2 (30 MVA)</v>
       </c>
       <c r="O18" t="str">
         <v/>
@@ -2998,13 +3600,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>Konsumen KTT PENDO (35 MVA)</v>
+        <v>KTT PENDO</v>
       </c>
       <c r="C19" t="str">
         <v>KTT PENDO</v>
       </c>
       <c r="D19" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="E19" t="str">
         <v>Normal</v>
@@ -3034,7 +3636,7 @@
         <v>JBB</v>
       </c>
       <c r="N19" t="str">
-        <v>Konsumen Tegangan Tinggi PENDO</v>
+        <v>Konsumen Tegangan Tinggi PENDO (35 MVA)</v>
       </c>
       <c r="O19" t="str">
         <v/>
@@ -3051,13 +3653,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>Konsumen KTT PENI (40 MVA)</v>
+        <v>KTT PENI</v>
       </c>
       <c r="C20" t="str">
         <v>KTT PENI</v>
       </c>
       <c r="D20" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="E20" t="str">
         <v>Normal</v>
@@ -3087,16 +3689,16 @@
         <v>JBB</v>
       </c>
       <c r="N20" t="str">
-        <v>Konsumen Tegangan Tinggi PENI Chandra Asri</v>
+        <v>Konsumen Tegangan Tinggi PENI Chandra Asri (40 MVA, Memiliki Kerawanan #3)</v>
       </c>
       <c r="O20" t="str">
-        <v/>
+        <v>Potensi kendala operasional saat gangguan ruas single phi.</v>
       </c>
       <c r="P20" t="str">
-        <v/>
+        <v>Jadwal pemeliharaan selaras dengan turn-around pabrik.</v>
       </c>
       <c r="Q20" t="str">
-        <v/>
+        <v>Usulan perkuatan sistem suplai transmisi.</v>
       </c>
     </row>
     <row r="21">
@@ -3104,13 +3706,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>Konsumen KTT LCI (115 MVA)</v>
+        <v>KTT LCI</v>
       </c>
       <c r="C21" t="str">
         <v>KTT LCI</v>
       </c>
       <c r="D21" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="E21" t="str">
         <v>Normal</v>
@@ -3140,7 +3742,7 @@
         <v>JBB</v>
       </c>
       <c r="N21" t="str">
-        <v>Konsumen KTT LCI</v>
+        <v>Konsumen KTT LCI (115 MVA, Disuplai 2 Sirkit dengan 2 PMT CB)</v>
       </c>
       <c r="O21" t="str">
         <v/>
@@ -3157,13 +3759,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>Konsumen KTT MCCI (40 MVA)</v>
+        <v>KTT MCCI</v>
       </c>
       <c r="C22" t="str">
         <v>KTT MCCI</v>
       </c>
       <c r="D22" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="E22" t="str">
         <v>Normal</v>
@@ -3193,7 +3795,7 @@
         <v>JBB</v>
       </c>
       <c r="N22" t="str">
-        <v>Konsumen KTT MCCI</v>
+        <v>Konsumen Tegangan Tinggi MCCI (40 MVA)</v>
       </c>
       <c r="O22" t="str">
         <v/>
@@ -3210,13 +3812,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>Konsumen KTT MTSUI (31 MVA)</v>
+        <v>KTT MTSUI</v>
       </c>
       <c r="C23" t="str">
         <v>KTT MTSUI</v>
       </c>
       <c r="D23" t="str">
-        <v>Beban</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="E23" t="str">
         <v>Normal</v>
@@ -3246,7 +3848,7 @@
         <v>JBB</v>
       </c>
       <c r="N23" t="str">
-        <v>Konsumen KTT Mitsui</v>
+        <v>Konsumen Tegangan Tinggi Mitsui (31 MVA, Terhubung ke GI MTSUI)</v>
       </c>
       <c r="O23" t="str">
         <v/>
@@ -3255,19 +3857,291 @@
         <v/>
       </c>
       <c r="Q23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Trafo Distribusi SRLYA</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Trafo SRLYA</v>
+      </c>
+      <c r="D24" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="F24" t="str">
+        <v>60 MVA</v>
+      </c>
+      <c r="G24">
+        <v>2</v>
+      </c>
+      <c r="H24" t="str">
+        <v>150/20 kV</v>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v>Banten</v>
+      </c>
+      <c r="M24" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Trafo distribusi lokal 150/20 kV Suralaya</v>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Trafo Distribusi CLBRU</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Trafo CLBRU</v>
+      </c>
+      <c r="D25" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="F25" t="str">
+        <v>60 MVA</v>
+      </c>
+      <c r="G25">
+        <v>2</v>
+      </c>
+      <c r="H25" t="str">
+        <v>150/20 kV</v>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v>Banten</v>
+      </c>
+      <c r="M25" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Trafo distribusi lokal 150/20 kV Cilegon Baru</v>
+      </c>
+      <c r="O25" t="str">
+        <v/>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Trafo Distribusi CLGON</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Trafo CLGON</v>
+      </c>
+      <c r="D26" t="str">
+        <v>trafo_distribusi</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="F26" t="str">
+        <v>60 MVA</v>
+      </c>
+      <c r="G26">
+        <v>3</v>
+      </c>
+      <c r="H26" t="str">
+        <v>150/20 kV</v>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v>Banten</v>
+      </c>
+      <c r="M26" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Trafo distribusi lokal 150/20 kV Cilegon Lama</v>
+      </c>
+      <c r="O26" t="str">
+        <v/>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>KSTEL</v>
+      </c>
+      <c r="C27" t="str">
+        <v>KSTEL</v>
+      </c>
+      <c r="D27" t="str">
+        <v>cb</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27">
+        <v>3</v>
+      </c>
+      <c r="H27" t="str">
+        <v>150 kV</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v>Banten</v>
+      </c>
+      <c r="M27" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Bay Rencana Konsumen Krakatau Steel (KSTEL) Garis Putus-putus</v>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>POSCO</v>
+      </c>
+      <c r="C28" t="str">
+        <v>POSCO</v>
+      </c>
+      <c r="D28" t="str">
+        <v>cb</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28">
+        <v>3</v>
+      </c>
+      <c r="H28" t="str">
+        <v>150 kV</v>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <v>Banten</v>
+      </c>
+      <c r="M28" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="N28" t="str">
+        <v>Bay Rencana Konsumen Krakatau Posco (POSCO) Garis Putus-putus</v>
+      </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q28"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E7"/>
+  <cols>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="48.83203125" customWidth="1"/>
+    <col min="4" max="4" width="55.83203125" customWidth="1"/>
+    <col min="5" max="5" width="45.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3288,150 +4162,127 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Peralatan (1)</v>
+        <v>1. Pembangkit / Generator</v>
       </c>
       <c r="B2" t="str">
-        <v>Generator / Pembangkit</v>
+        <v>generator</v>
       </c>
       <c r="C2" t="str">
-        <v>Lingkaran Hijau dengan Gelombang Sinus AC (~)</v>
+        <v>Lingkaran Hijau + Simbol Gelombang AC (~)</v>
       </c>
       <c r="D2" t="str">
-        <v>Titik hulu pembangkit listrik utama (PLTU, PLTA, PLTG, PLTGU).</v>
+        <v>Digunakan untuk merepresentasikan sumber daya pembangkitan (PLTU, PLTGU, PLTA, dll). Pada diagram terletak di bagian paling atas (Unit 3).</v>
       </c>
       <c r="E2" t="str">
-        <v>PLTU Suralaya Unit 3 (600 MW)</v>
+        <v>PLTU Suralaya Unit 3, PLTGU Muara Karang Unit 1-3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Peralatan (2)</v>
+        <v>2. Trafo Generator (GSUT)</v>
       </c>
       <c r="B3" t="str">
-        <v>Trafo Generator (GSUT)</v>
+        <v>trafo_generator</v>
       </c>
       <c r="C3" t="str">
-        <v>2 Lingkaran Interlocking (Atas: Hijau sisi Gen, Bawah: Merah sisi GI)</v>
+        <v>Dua Cincin Bertaut: Atas Hijau (Generator), Bawah Merah (Tegangan Tinggi)</v>
       </c>
       <c r="D3" t="str">
-        <v>Trafo penaik tegangan generator (Generator Step-Up) dari 15-20 kV ke tegangan tinggi GI (150/500 kV).</v>
+        <v>Digunakan untuk menaikkan tegangan dari generator pembangkit ke tegangan sistem transmisi (Generator Step-Up Transformer / GSUT).</v>
       </c>
       <c r="E3" t="str">
-        <v>Bay Pembangkit ke Busbar GI</v>
+        <v>Trafo Step-Up PLTU Unit 3 ke Busbar 150 kV SRLYA</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Switching (3)</v>
+        <v>3. Circuit Breaker (PMT)</v>
       </c>
       <c r="B4" t="str">
-        <v>CB / PMT (Pemutus Tenaga)</v>
+        <v>cb</v>
       </c>
       <c r="C4" t="str">
-        <v>Balok / Persegi Panjang Solid Merah Tegak dengan garis terminal</v>
+        <v>Balok Persegi Merah Solid pada Jalur Penghantar</v>
       </c>
       <c r="D4" t="str">
-        <v>Circuit Breaker pada bay pengirim dan penerima GI ke GI untuk memutus beban dan gangguan arus pendek.</v>
+        <v>Pemutus Tenaga (PMT / Circuit Breaker) yang diletakkan pada bay pengirim maupun penerima GI ke GI untuk memutus arus gangguan.</v>
       </c>
       <c r="E4" t="str">
-        <v>Bay Line, Bay IBT, Bay Trafo, Bay Generator</v>
+        <v>Semua bay outgoing/incoming SUTT 150 kV, bay trafo, dan bay IBT</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Peralatan (4)</v>
+        <v>4. Interbus Transformer (IBT)</v>
       </c>
       <c r="B5" t="str">
-        <v>IBT (Interbus Transformer)</v>
+        <v>ibt</v>
       </c>
       <c r="C5" t="str">
-        <v>3 Lingkaran Bertumpuk (Atas Biru 500kV, Kiri Merah 150kV, Kanan Kuning 33kV)</v>
+        <v>Tiga Cincin Bertaut: Atas Biru (500 kV), Kiri Merah (150 kV), Kanan Kuning (Tertiary 33/20 kV)</v>
       </c>
       <c r="D5" t="str">
-        <v>Trafo interkoneksi sistem transmisi tegangan ekstra tinggi (500/150 kV atau 275/150 kV).</v>
+        <v>Transformator Daya Besar (3 Winding) penghubung antar grid tegangan ekstra tinggi 500 kV atau 275 kV ke tegangan transmisi 150 kV.</v>
       </c>
       <c r="E5" t="str">
-        <v>IBT 1 &amp; 2 Suralaya (250 MVA), IBT 4 Cilegon (500 MVA)</v>
+        <v>IBT 1 Suralaya (500/150 kV), IBT 2 Suralaya Baru, IBT 4 Cilegon Baru</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Peralatan (5)</v>
+        <v>5. Trafo Distribusi / KTT</v>
       </c>
       <c r="B6" t="str">
-        <v>Trafo Distribusi</v>
+        <v>trafo_distribusi</v>
       </c>
       <c r="C6" t="str">
-        <v>2 Lingkaran Interlocking (Atas: Merah 150kV, Bawah: Kuning 20kV / 70kV)</v>
+        <v>Dua Cincin Bertaut: Atas Merah (150 kV), Bawah Kuning (20 kV / 70 kV)</v>
       </c>
       <c r="D6" t="str">
-        <v>Trafo step-down daya di Gardu Induk yang menurunkan tegangan dari 150 kV ke 70 kV atau 20 kV.</v>
+        <v>Transformator penurun tegangan dari transmisi 150 kV ke tegangan menengah 20 kV (atau 70 kV) untuk melayani gardu distribusi &amp; konsumen tegangan tinggi (KTT).</v>
       </c>
       <c r="E6" t="str">
-        <v>Trafo 150/20 kV GI Distribusi / Feeder KTT</v>
+        <v>Trafo KTT SLFDO-1 (78 MVA), KTT PENI (40 MVA), KTT LCI (115 MVA), KTT MTSUI</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Peralatan (6)</v>
+        <v>6. Busbar (Rel Konduktor)</v>
       </c>
       <c r="B7" t="str">
-        <v>Busbar</v>
+        <v>busbar</v>
       </c>
       <c r="C7" t="str">
-        <v>Batang Rel Horizontal Tebal (Cyan/Biru)</v>
+        <v>Garis Horisontal Tebal: Biru (500 kV) atau Merah (150 kV)</v>
       </c>
       <c r="D7" t="str">
-        <v>Batang konduktor utama di Gardu Induk (GI / GITET) yang mengumpulkan dan membagikan daya listrik.</v>
+        <v>Rel konduktor pengumpul daya listrik di gardu induk. Dapat diset 'Normal' atau 'Panjang (Wide Busbar)' untuk membentang di atas beberapa bay.</v>
       </c>
       <c r="E7" t="str">
-        <v>Suralaya Baru (500 kV), GI SRLYA 150 kV, GI CLBRU 150 kV</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Peralatan (7)</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Beban</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Segitiga Terbalik (∇) Kuning Emas dengan terminal bulatan di atas</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Simbol resmi beban listrik konsumen industri KTT (Konsumen Tegangan Tinggi) atau feeder beban.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>KTT SLFDO-1 (78 MVA), KTT PENI (40 MVA), KTT LCI (115 MVA)</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Peralatan (8)</v>
-      </c>
-      <c r="B9" t="str">
-        <v>PHT (Penghantar)</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Kapsul Saluran Transmisi dengan dua bulatan terminal di ujung</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Saluran udara/kabel transmisi tenaga listrik penghubung antar gardu induk.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>PHT Suralaya - Salira Indah, PHT Suralaya - PENI</v>
+        <v>Rel 500 kV Suralaya Baru, Rel 150 kV SRLYA (Wide Busbar), Rel 150 kV CLBRU</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
+  <cols>
+    <col min="1" max="1" width="5.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="35.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
+    <col min="8" max="8" width="40.83203125" customWidth="1"/>
+    <col min="9" max="9" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3444,18 +4295,21 @@
         <v>Subsistem</v>
       </c>
       <c r="D1" t="str">
+        <v>Peralatan Terdampak</v>
+      </c>
+      <c r="E1" t="str">
         <v>UIT</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Kondisi / Permasalahan</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Dampak</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Mitigasi</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Usulan / Solusi</v>
       </c>
     </row>
@@ -3467,27 +4321,30 @@
         <v>1&amp;2</v>
       </c>
       <c r="C2" t="str">
-        <v>Subsistem Suralaya Unit #3 - Suralaya 1,2 – Cilegon 4</v>
+        <v>Suralaya - Cilegon</v>
       </c>
       <c r="D2" t="str">
-        <v>JBB</v>
+        <v>IBT 1 Suralaya &amp; IBT 2 Suralaya Baru (500/150 kV)</v>
       </c>
       <c r="E2" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="F2" t="str">
         <v>Pembebanan IBT–1,2 Suralaya tidak memenuhi kriteria N–1 saat PLTU Suralaya unit–3 tidak beroperasi dan IBT–4 Cilegon masuk sub sistem Cilegon.</v>
       </c>
-      <c r="F2" t="str" xml:space="preserve">
+      <c r="G2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Pemeliharaan IBT sulit dilakukan.
 2. Pertumbuhan beban menjadi terhambat.
 3. Terjadi pemadaman apabila trip salah satu IBT di Suralaya.</v>
       </c>
-      <c r="G2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW (Berdasarkan buku DS Tahun 2025).
-2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan total target sebesar 137 MW (Berdasarkan buku DS Tahun 2025).
-3. Pemeliharaan IBT saat beban rendah dan pada saat PLTU Suralaya Unit–3 beroperasi.</v>
-      </c>
       <c r="H2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW.
+2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan target total 137 MW.
+3. Pemeliharaan IBT saat beban rendah dan Unit 3 beroperasi.</v>
+      </c>
+      <c r="I2" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2025.</v>
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2025/2026.</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -3498,26 +4355,27 @@
         <v>2</v>
       </c>
       <c r="C3" t="str">
-        <v>Subsistem Suralaya Unit #3 - Suralaya 1,2 – Cilegon 4</v>
+        <v>Suralaya - Cilegon</v>
       </c>
       <c r="D3" t="str">
-        <v>JBB</v>
+        <v>IBT 4 Cilegon Baru (500/150 kV)</v>
       </c>
       <c r="E3" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="F3" t="str">
         <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA sedangkan IBT #4 Cilegon 500 MVA).</v>
       </c>
-      <c r="F3" t="str" xml:space="preserve">
+      <c r="G3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Ketidakseimbangan beban antara IBT Suralaya dan IBT Cilegon.
-2. Kondisi N–1–1 (IBT Suralaya dan IBT Cilegon) berdampak overload pada IBT Suralaya yang beroperasi.</v>
-      </c>
-      <c r="G3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW (Berdasarkan buku DS Tahun 2025).
-2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan total target sebesar 137 MW (Berdasarkan buku DS Tahun 2025).
-3. Pemeliharaan IBT saat beban rendah dan pada saat PLTU Suralaya Unit–3 beroperasi.</v>
-      </c>
-      <c r="H3" t="str" xml:space="preserve">
+2. Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Optimalisasi transfer trip dan defense scheme antar GI.</v>
+      </c>
+      <c r="I3" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2026.</v>
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA.</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -3528,30 +4386,33 @@
         <v>3</v>
       </c>
       <c r="C4" t="str">
-        <v>Subsistem Suralaya Unit #3 - Suralaya 1,2 – Cilegon 4</v>
+        <v>Suralaya - Cilegon</v>
       </c>
       <c r="D4" t="str">
-        <v>JBB</v>
+        <v>Ruas SUTT Suralaya–PENI, Suralaya–MCCI, MCCI–Cilegon, PENI–Mitsui–Cilegon</v>
       </c>
       <c r="E4" t="str">
+        <v>JBB</v>
+      </c>
+      <c r="F4" t="str">
         <v>Ruas Penghantar Suralaya–MCCI–Cilegon dan Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
       </c>
-      <c r="F4" t="str" xml:space="preserve">
+      <c r="G4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Pemeliharaan Penghantar menjadi sulit dilakukan.
 2. Terjadi pemadaman apabila terdapat gangguan N–1–1.</v>
       </c>
-      <c r="G4" t="str" xml:space="preserve">
+      <c r="H4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Pemeliharaan Penghantar menyesuaikan jadwal dari KTT.
 2. Pengaturan konfigurasi jaringan saat pemeliharaan untuk mengurangi dampak padam.</v>
       </c>
-      <c r="H4" t="str" xml:space="preserve">
+      <c r="I4" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Menengah :
 Usulan Double phi pada ruas Suralaya s.d Cilegon Lama (Kajian belum ada). Diusulkan COD Tahun 2030.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(sld): restore authentic topology, eliminate phantom nodes, and correctly render 5 PLN equipment symbols
</commit_message>
<xml_diff>
--- a/peta-kerawanan/dist/template_kerawanan_subsistem_suralaya_cilegon.xlsx
+++ b/peta-kerawanan/dist/template_kerawanan_subsistem_suralaya_cilegon.xlsx
@@ -400,34 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y28"/>
-  <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="38.83203125" customWidth="1"/>
-    <col min="4" max="4" width="26.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="16.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" customWidth="1"/>
-    <col min="15" max="15" width="16.83203125" customWidth="1"/>
-    <col min="16" max="16" width="20.83203125" customWidth="1"/>
-    <col min="17" max="17" width="24.83203125" customWidth="1"/>
-    <col min="18" max="18" width="24.83203125" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" customWidth="1"/>
-    <col min="20" max="20" width="22.83203125" customWidth="1"/>
-    <col min="21" max="21" width="10.83203125" customWidth="1"/>
-    <col min="22" max="22" width="45.83203125" customWidth="1"/>
-    <col min="23" max="23" width="35.83203125" customWidth="1"/>
-    <col min="24" max="24" width="35.83203125" customWidth="1"/>
-    <col min="25" max="25" width="35.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:Y21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -506,27 +479,27 @@
         <v>Usulan / Solusi</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>1&amp;2</v>
       </c>
       <c r="C2" t="str">
-        <v>Bay Evakuasi PLTU Suralaya Unit 3</v>
+        <v>Bay IBT 2 Suralaya Baru (500/150 kV)</v>
       </c>
       <c r="D2" t="str">
-        <v>Bay Generator &amp; GSUT</v>
+        <v>Bay IBT</v>
       </c>
       <c r="E2" t="str">
-        <v>trafo_generator</v>
+        <v>IBT</v>
       </c>
       <c r="F2" t="str">
-        <v>Unit 3</v>
+        <v>Suralaya Baru</v>
       </c>
       <c r="G2" t="str">
-        <v>generator</v>
+        <v>Busbar</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -535,13 +508,13 @@
         <v>SRLYA</v>
       </c>
       <c r="J2" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="K2">
         <v>1</v>
       </c>
       <c r="L2" t="str">
-        <v>500 kV</v>
+        <v>500/150 kV</v>
       </c>
       <c r="M2">
         <v>1</v>
@@ -553,16 +526,16 @@
         <v>Beroperasi</v>
       </c>
       <c r="P2" t="str">
-        <v>Normal</v>
+        <v>Sangat Rawan</v>
       </c>
       <c r="Q2">
-        <v>60</v>
+        <v>88</v>
       </c>
       <c r="R2" t="str">
         <v/>
       </c>
       <c r="S2">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="T2" t="str">
         <v>Banten - Cilegon</v>
@@ -571,16 +544,21 @@
         <v>JBB</v>
       </c>
       <c r="V2" t="str">
-        <v>Bay Pembangkit Unit 3: 1. Generator (Hijau), 2. Trafo GSUT (Hijau-Merah), 3. CB PMT (Balok Merah)</v>
-      </c>
-      <c r="W2" t="str">
-        <v/>
-      </c>
-      <c r="X2" t="str">
-        <v/>
-      </c>
-      <c r="Y2" t="str">
-        <v/>
+        <v>Pembebanan IBT–1,2 Suralaya tidak memenuhi kriteria N–1 saat PLTU Suralaya unit–3 tidak beroperasi dan IBT–4 Cilegon masuk sub sistem Cilegon.</v>
+      </c>
+      <c r="W2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Pemeliharaan IBT sulit dilakukan.
+2. Pertumbuhan beban menjadi terhambat.
+3. Terjadi pemadaman apabila trip salah satu IBT di Suralaya.</v>
+      </c>
+      <c r="X2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW.
+2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan total target sebesar 137 MW.
+3. Pemeliharaan IBT saat beban rendah.</v>
+      </c>
+      <c r="Y2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Jangka Pendek :
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2025.</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -591,19 +569,19 @@
         <v>1&amp;2</v>
       </c>
       <c r="C3" t="str">
-        <v>Bay IBT 2 Suralaya Baru (500/150 kV)</v>
+        <v>Bay IBT 1 Suralaya (500/150 kV)</v>
       </c>
       <c r="D3" t="str">
-        <v>Bay Interbus Transformer</v>
+        <v>Bay IBT</v>
       </c>
       <c r="E3" t="str">
-        <v>ibt</v>
+        <v>IBT</v>
       </c>
       <c r="F3" t="str">
-        <v>Suralaya Baru</v>
+        <v>Suralaya</v>
       </c>
       <c r="G3" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -612,7 +590,7 @@
         <v>SRLYA</v>
       </c>
       <c r="J3" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="K3">
         <v>1</v>
@@ -633,7 +611,7 @@
         <v>Sangat Rawan</v>
       </c>
       <c r="Q3">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="R3" t="str">
         <v/>
@@ -648,21 +626,19 @@
         <v>JBB</v>
       </c>
       <c r="V3" t="str">
-        <v>Pembebanan IBT–1,2 Suralaya tidak memenuhi kriteria N–1 saat PLTU Suralaya unit–3 tidak beroperasi dan IBT–4 Cilegon masuk sub sistem Cilegon.</v>
+        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA sedangkan IBT #4 Cilegon 500 MVA).</v>
       </c>
       <c r="W3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Pemeliharaan IBT sulit dilakukan.
-2. Pertumbuhan beban menjadi terhambat.
-3. Terjadi pemadaman apabila trip salah satu IBT di Suralaya.</v>
+        <v xml:space="preserve">1. Ketidakseimbangan beban antara IBT Suralaya dan IBT Cilegon.
+2. Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
       </c>
       <c r="X3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW.
-2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan target total 137 MW.
-3. Pemeliharaan IBT saat beban rendah.</v>
+        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya.
+2. Pemeliharaan IBT saat beban rendah.</v>
       </c>
       <c r="Y3" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD Tahun 2025.</v>
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2026.</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -670,31 +646,31 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>1&amp;2</v>
+        <v>2</v>
       </c>
       <c r="C4" t="str">
-        <v>Bay IBT 1 Suralaya (500/150 kV)</v>
+        <v>Bay IBT 4 Cilegon Baru (500/150 kV)</v>
       </c>
       <c r="D4" t="str">
-        <v>Bay Interbus Transformer</v>
+        <v>Bay IBT</v>
       </c>
       <c r="E4" t="str">
-        <v>ibt</v>
+        <v>IBT</v>
       </c>
       <c r="F4" t="str">
-        <v>Suralaya</v>
+        <v>Cilegon Baru</v>
       </c>
       <c r="G4" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4" t="str">
-        <v>SRLYA</v>
+        <v>CLBRU</v>
       </c>
       <c r="J4" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="K4">
         <v>1</v>
@@ -715,7 +691,7 @@
         <v>Sangat Rawan</v>
       </c>
       <c r="Q4">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="R4" t="str">
         <v/>
@@ -730,57 +706,55 @@
         <v>JBB</v>
       </c>
       <c r="V4" t="str">
-        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA sedangkan IBT #4 Cilegon 500 MVA).</v>
-      </c>
-      <c r="W4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Ketidakseimbangan beban antara IBT Suralaya dan IBT Cilegon.
-2. Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
-      </c>
-      <c r="X4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW.
-2. Pemeliharaan IBT saat beban rendah dan Unit 3 beroperasi.</v>
+        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama.</v>
+      </c>
+      <c r="W4" t="str">
+        <v>Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
+      </c>
+      <c r="X4" t="str">
+        <v>Optimalisasi transfer trip dan defense scheme antar GI.</v>
       </c>
       <c r="Y4" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD Tahun 2026.</v>
-      </c>
-    </row>
-    <row r="5" xml:space="preserve">
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA.</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="C5" t="str">
-        <v>Bay IBT 4 Cilegon Baru (500/150 kV)</v>
+        <v>Bay Evakuasi Unit 3 PLTU Suralaya</v>
       </c>
       <c r="D5" t="str">
-        <v>Bay Interbus Transformer</v>
+        <v>Bay Generator</v>
       </c>
       <c r="E5" t="str">
-        <v>ibt</v>
+        <v>Trafo Generator</v>
       </c>
       <c r="F5" t="str">
-        <v>Cilegon Baru</v>
+        <v>Unit 3</v>
       </c>
       <c r="G5" t="str">
-        <v>busbar</v>
+        <v>Pembangkit</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
       <c r="I5" t="str">
-        <v>CLBRU</v>
+        <v>SRLYA</v>
       </c>
       <c r="J5" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="K5">
         <v>1</v>
       </c>
       <c r="L5" t="str">
-        <v>500/150 kV</v>
+        <v>500 kV</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -792,16 +766,16 @@
         <v>Beroperasi</v>
       </c>
       <c r="P5" t="str">
-        <v>Sangat Rawan</v>
+        <v>Normal</v>
       </c>
       <c r="Q5">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="R5" t="str">
         <v/>
       </c>
       <c r="S5">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="T5" t="str">
         <v>Banten - Cilegon</v>
@@ -810,17 +784,16 @@
         <v>JBB</v>
       </c>
       <c r="V5" t="str">
-        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #4 Cilegon 500 MVA sedangkan IBT #1,2 Suralaya 250 MVA).</v>
+        <v>Evakuasi daya PLTU Suralaya Unit 3 (1. Pembangkit, 2. Trafo Step-Up, 3. CB).</v>
       </c>
       <c r="W5" t="str">
-        <v>Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
+        <v/>
       </c>
       <c r="X5" t="str">
-        <v>Optimalisasi transfer trip dan defense scheme antar GI.</v>
-      </c>
-      <c r="Y5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. COD Tahun 2026.</v>
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -831,19 +804,19 @@
         <v/>
       </c>
       <c r="C6" t="str">
-        <v>SUTT 150 kV SRLYA - SLRDA</v>
+        <v>Suralaya - Salira Indah (Sirkit 1)</v>
       </c>
       <c r="D6" t="str">
-        <v>Saluran Udara (SUTT)</v>
+        <v>PHT</v>
       </c>
       <c r="E6" t="str">
-        <v>cb</v>
+        <v>PHT</v>
       </c>
       <c r="F6" t="str">
         <v>SRLYA</v>
       </c>
       <c r="G6" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -852,7 +825,7 @@
         <v>SLRDA</v>
       </c>
       <c r="J6" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="K6">
         <v>2</v>
@@ -861,7 +834,7 @@
         <v>150 kV</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N6">
         <v>1</v>
@@ -873,13 +846,13 @@
         <v>Normal</v>
       </c>
       <c r="Q6">
-        <v>54</v>
-      </c>
-      <c r="R6" t="str">
-        <v/>
+        <v>52</v>
+      </c>
+      <c r="R6">
+        <v>48</v>
       </c>
       <c r="S6">
-        <v>14.2</v>
+        <v>12.5</v>
       </c>
       <c r="T6" t="str">
         <v>Banten - Cilegon</v>
@@ -908,28 +881,28 @@
         <v/>
       </c>
       <c r="C7" t="str">
-        <v>SUTT 150 kV SRLYA - PENDO</v>
+        <v>Suralaya - Salira Indah (Sirkit 2)</v>
       </c>
       <c r="D7" t="str">
-        <v>Saluran Udara (SUTT)</v>
+        <v>PHT</v>
       </c>
       <c r="E7" t="str">
-        <v>cb</v>
+        <v>PHT</v>
       </c>
       <c r="F7" t="str">
         <v>SRLYA</v>
       </c>
       <c r="G7" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7" t="str">
-        <v>PENDO</v>
+        <v>SLRDA</v>
       </c>
       <c r="J7" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="K7">
         <v>2</v>
@@ -938,10 +911,10 @@
         <v>150 kV</v>
       </c>
       <c r="M7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O7" t="str">
         <v>Beroperasi</v>
@@ -950,13 +923,13 @@
         <v>Normal</v>
       </c>
       <c r="Q7">
+        <v>52</v>
+      </c>
+      <c r="R7">
         <v>48</v>
       </c>
-      <c r="R7" t="str">
-        <v/>
-      </c>
       <c r="S7">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="T7" t="str">
         <v>Banten - Cilegon</v>
@@ -985,19 +958,19 @@
         <v/>
       </c>
       <c r="C8" t="str">
-        <v>SUTT 150 kV Tie Line SLRDA - PENDO</v>
+        <v>Salira Indah - Pendo</v>
       </c>
       <c r="D8" t="str">
-        <v>Tie Line Interkoneksi</v>
+        <v>PHT</v>
       </c>
       <c r="E8" t="str">
-        <v>cb</v>
+        <v>PHT</v>
       </c>
       <c r="F8" t="str">
         <v>SLRDA</v>
       </c>
       <c r="G8" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H8">
         <v>2</v>
@@ -1006,7 +979,7 @@
         <v>PENDO</v>
       </c>
       <c r="J8" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="K8">
         <v>2</v>
@@ -1027,13 +1000,13 @@
         <v>Normal</v>
       </c>
       <c r="Q8">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="R8" t="str">
         <v/>
       </c>
       <c r="S8">
-        <v>6.4</v>
+        <v>8.4</v>
       </c>
       <c r="T8" t="str">
         <v>Banten - Cilegon</v>
@@ -1042,7 +1015,7 @@
         <v>JBB</v>
       </c>
       <c r="V8" t="str">
-        <v>Interkoneksi antar bay busbar Salira Indah (SLRDA) dan Pendo (PENDO) di Tier 2.</v>
+        <v/>
       </c>
       <c r="W8" t="str">
         <v/>
@@ -1054,7 +1027,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" xml:space="preserve">
+    <row r="9">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1062,19 +1035,19 @@
         <v>3</v>
       </c>
       <c r="C9" t="str">
-        <v>SUTT 150 kV SRLYA - PENI</v>
+        <v>Suralaya - Chandra Asri (PENI)</v>
       </c>
       <c r="D9" t="str">
-        <v>Saluran Udara (SUTT)</v>
+        <v>PHT</v>
       </c>
       <c r="E9" t="str">
-        <v>cb</v>
+        <v>PHT</v>
       </c>
       <c r="F9" t="str">
         <v>SRLYA</v>
       </c>
       <c r="G9" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -1083,7 +1056,7 @@
         <v>PENI</v>
       </c>
       <c r="J9" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="K9">
         <v>2</v>
@@ -1104,13 +1077,13 @@
         <v>N-1</v>
       </c>
       <c r="Q9">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="R9" t="str">
         <v/>
       </c>
       <c r="S9">
-        <v>18.5</v>
+        <v>15.2</v>
       </c>
       <c r="T9" t="str">
         <v>Banten - Cilegon</v>
@@ -1119,22 +1092,19 @@
         <v>JBB</v>
       </c>
       <c r="V9" t="str">
-        <v>Ruas Penghantar Suralaya–MCCI–Cilegon dan Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
-      </c>
-      <c r="W9" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Pemeliharaan Penghantar menjadi sulit dilakukan.
-2. Terjadi pemadaman apabila terdapat gangguan N–1–1.</v>
-      </c>
-      <c r="X9" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Pemeliharaan Penghantar menyesuaikan jadwal dari KTT.
-2. Pengaturan konfigurasi jaringan saat pemeliharaan untuk mengurangi dampak padam.</v>
-      </c>
-      <c r="Y9" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jangka Menengah :
-Usulan Double phi pada ruas Suralaya s.d Cilegon Lama (Kajian belum ada). Diusulkan COD Tahun 2030.</v>
-      </c>
-    </row>
-    <row r="10" xml:space="preserve">
+        <v>Ruas Penghantar Suralaya-PENI masih single phi.</v>
+      </c>
+      <c r="W9" t="str">
+        <v>Pemadaman apabila trip saat pemeliharaan KTT.</v>
+      </c>
+      <c r="X9" t="str">
+        <v>Penyesuaian jadwal pemeliharaan.</v>
+      </c>
+      <c r="Y9" t="str">
+        <v>Double phi COD 2030.</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1142,19 +1112,19 @@
         <v>3</v>
       </c>
       <c r="C10" t="str">
-        <v>SUTT 150 kV SRLYA - MCCI5</v>
+        <v>Suralaya - MCCI</v>
       </c>
       <c r="D10" t="str">
-        <v>Saluran Udara (SUTT)</v>
+        <v>PHT</v>
       </c>
       <c r="E10" t="str">
-        <v>cb</v>
+        <v>PHT</v>
       </c>
       <c r="F10" t="str">
         <v>SRLYA</v>
       </c>
       <c r="G10" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -1163,7 +1133,7 @@
         <v>MCCI5</v>
       </c>
       <c r="J10" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="K10">
         <v>2</v>
@@ -1184,13 +1154,13 @@
         <v>N-1</v>
       </c>
       <c r="Q10">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="R10" t="str">
         <v/>
       </c>
       <c r="S10">
-        <v>16.3</v>
+        <v>16.8</v>
       </c>
       <c r="T10" t="str">
         <v>Banten - Cilegon</v>
@@ -1199,60 +1169,57 @@
         <v>JBB</v>
       </c>
       <c r="V10" t="str">
-        <v>Ruas Penghantar Suralaya–MCCI–Cilegon dan Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
-      </c>
-      <c r="W10" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Pemeliharaan Penghantar menjadi sulit dilakukan.
-2. Terjadi pemadaman apabila terdapat gangguan N–1–1.</v>
-      </c>
-      <c r="X10" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Pemeliharaan Penghantar menyesuaikan jadwal dari KTT.
-2. Pengaturan konfigurasi jaringan saat pemeliharaan.</v>
-      </c>
-      <c r="Y10" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jangka Menengah :
-Usulan Double phi pada ruas Suralaya s.d Cilegon Lama. COD Tahun 2030.</v>
-      </c>
-    </row>
-    <row r="11" xml:space="preserve">
+        <v>Ruas Penghantar Suralaya-MCCI-Cilegon masih single phi.</v>
+      </c>
+      <c r="W10" t="str">
+        <v>Pemadaman apabila terjadi trip.</v>
+      </c>
+      <c r="X10" t="str">
+        <v>Penyesuaian jadwal pemeliharaan dari KTT.</v>
+      </c>
+      <c r="Y10" t="str">
+        <v>Usulan double phi ruas Suralaya s.d Cilegon Lama.</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="C11" t="str">
-        <v>SUTT 150 kV PENI - MTSUI</v>
+        <v>Cilegon Baru - Cilegon Lama (Sirkit 1)</v>
       </c>
       <c r="D11" t="str">
-        <v>Saluran Udara (SUTT)</v>
+        <v>PHT</v>
       </c>
       <c r="E11" t="str">
-        <v>cb</v>
+        <v>PHT</v>
       </c>
       <c r="F11" t="str">
-        <v>PENI</v>
+        <v>CLBRU</v>
       </c>
       <c r="G11" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11" t="str">
+        <v>CLGON</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K11">
         <v>2</v>
-      </c>
-      <c r="I11" t="str">
-        <v>MTSUI</v>
-      </c>
-      <c r="J11" t="str">
-        <v>busbar</v>
-      </c>
-      <c r="K11">
-        <v>3</v>
       </c>
       <c r="L11" t="str">
         <v>150 kV</v>
       </c>
       <c r="M11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N11">
         <v>1</v>
@@ -1261,16 +1228,16 @@
         <v>Beroperasi</v>
       </c>
       <c r="P11" t="str">
-        <v>N-1</v>
+        <v>Normal</v>
       </c>
       <c r="Q11">
-        <v>68</v>
-      </c>
-      <c r="R11" t="str">
-        <v/>
+        <v>54</v>
+      </c>
+      <c r="R11">
+        <v>50</v>
       </c>
       <c r="S11">
-        <v>8.7</v>
+        <v>9.2</v>
       </c>
       <c r="T11" t="str">
         <v>Banten - Cilegon</v>
@@ -1279,18 +1246,16 @@
         <v>JBB</v>
       </c>
       <c r="V11" t="str">
-        <v>Ruas Penghantar Suralaya–MCCI–Cilegon dan Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
-      </c>
-      <c r="W11" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Pemeliharaan Penghantar menjadi sulit dilakukan.
-2. Terjadi pemadaman apabila terdapat gangguan N–1–1.</v>
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
       </c>
       <c r="X11" t="str">
-        <v>1. Pemeliharaan Penghantar menyesuaikan jadwal dari KTT.</v>
-      </c>
-      <c r="Y11" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jangka Menengah :
-Usulan Double phi pada ruas Suralaya s.d Cilegon Lama. COD Tahun 2030.</v>
+        <v/>
+      </c>
+      <c r="Y11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -1298,31 +1263,31 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="C12" t="str">
-        <v>SUTT 150 kV MCCI5 - CLGON</v>
+        <v>Cilegon Baru - Cilegon Lama (Sirkit 2)</v>
       </c>
       <c r="D12" t="str">
-        <v>Saluran Udara (SUTT)</v>
+        <v>PHT</v>
       </c>
       <c r="E12" t="str">
-        <v>cb</v>
+        <v>PHT</v>
       </c>
       <c r="F12" t="str">
-        <v>MCCI5</v>
+        <v>CLBRU</v>
       </c>
       <c r="G12" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12" t="str">
         <v>CLGON</v>
       </c>
       <c r="J12" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="K12">
         <v>2</v>
@@ -1331,25 +1296,25 @@
         <v>150 kV</v>
       </c>
       <c r="M12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" t="str">
         <v>Beroperasi</v>
       </c>
       <c r="P12" t="str">
-        <v>N-1</v>
+        <v>Normal</v>
       </c>
       <c r="Q12">
-        <v>65</v>
-      </c>
-      <c r="R12" t="str">
-        <v/>
+        <v>54</v>
+      </c>
+      <c r="R12">
+        <v>50</v>
       </c>
       <c r="S12">
-        <v>9.4</v>
+        <v>9.2</v>
       </c>
       <c r="T12" t="str">
         <v>Banten - Cilegon</v>
@@ -1358,16 +1323,16 @@
         <v>JBB</v>
       </c>
       <c r="V12" t="str">
-        <v>Ruas Penghantar Suralaya–MCCI–Cilegon dan Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
+        <v/>
       </c>
       <c r="W12" t="str">
-        <v>Pemadaman apabila trip saat pemeliharaan KTT.</v>
+        <v/>
       </c>
       <c r="X12" t="str">
-        <v>Penyesuaian jadwal pemeliharaan dari KTT.</v>
+        <v/>
       </c>
       <c r="Y12" t="str">
-        <v>Usulan double phi ruas Suralaya s.d Cilegon Lama. COD Tahun 2030.</v>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -1378,31 +1343,31 @@
         <v>3</v>
       </c>
       <c r="C13" t="str">
-        <v>SUTT 150 kV MTSUI - CLGON</v>
+        <v>Chandra Asri (PENI) - Mitsui (MTSUI)</v>
       </c>
       <c r="D13" t="str">
-        <v>Saluran Udara (SUTT)</v>
+        <v>PHT</v>
       </c>
       <c r="E13" t="str">
-        <v>cb</v>
+        <v>PHT</v>
       </c>
       <c r="F13" t="str">
+        <v>PENI</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H13">
+        <v>2</v>
+      </c>
+      <c r="I13" t="str">
         <v>MTSUI</v>
       </c>
-      <c r="G13" t="str">
-        <v>busbar</v>
-      </c>
-      <c r="H13">
+      <c r="J13" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="K13">
         <v>3</v>
-      </c>
-      <c r="I13" t="str">
-        <v>CLGON</v>
-      </c>
-      <c r="J13" t="str">
-        <v>busbar</v>
-      </c>
-      <c r="K13">
-        <v>2</v>
       </c>
       <c r="L13" t="str">
         <v>150 kV</v>
@@ -1420,13 +1385,13 @@
         <v>N-1</v>
       </c>
       <c r="Q13">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="R13" t="str">
         <v/>
       </c>
       <c r="S13">
-        <v>10.5</v>
+        <v>6.8</v>
       </c>
       <c r="T13" t="str">
         <v>Banten - Cilegon</v>
@@ -1435,16 +1400,16 @@
         <v>JBB</v>
       </c>
       <c r="V13" t="str">
-        <v>Ruas Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
+        <v>Ruas Peni-Mitsui-Cilegon masih single phi.</v>
       </c>
       <c r="W13" t="str">
-        <v>Pemadaman apabila terjadi gangguan N-1.</v>
+        <v>Pemadaman apabila trip.</v>
       </c>
       <c r="X13" t="str">
-        <v>Pengaturan konfigurasi jaringan sistem Banten.</v>
+        <v>Jadwal pemeliharaan KTT.</v>
       </c>
       <c r="Y13" t="str">
-        <v>Double phi ruas Suralaya s.d Cilegon Lama.</v>
+        <v>Usulan double phi COD 2030.</v>
       </c>
     </row>
     <row r="14">
@@ -1455,28 +1420,28 @@
         <v/>
       </c>
       <c r="C14" t="str">
-        <v>SUTT 150 kV CLBRU - CLGON Sirkit 1</v>
+        <v>Mitsui (MTSUI) - Cilegon Lama</v>
       </c>
       <c r="D14" t="str">
-        <v>Double Circuit Line 1</v>
+        <v>PHT</v>
       </c>
       <c r="E14" t="str">
-        <v>cb</v>
+        <v>PHT</v>
       </c>
       <c r="F14" t="str">
-        <v>CLBRU</v>
+        <v>MTSUI</v>
       </c>
       <c r="G14" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I14" t="str">
         <v>CLGON</v>
       </c>
       <c r="J14" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="K14">
         <v>2</v>
@@ -1485,7 +1450,7 @@
         <v>150 kV</v>
       </c>
       <c r="M14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14">
         <v>1</v>
@@ -1497,13 +1462,13 @@
         <v>Normal</v>
       </c>
       <c r="Q14">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="R14" t="str">
         <v/>
       </c>
       <c r="S14">
-        <v>11.2</v>
+        <v>5.4</v>
       </c>
       <c r="T14" t="str">
         <v>Banten - Cilegon</v>
@@ -1512,7 +1477,7 @@
         <v>JBB</v>
       </c>
       <c r="V14" t="str">
-        <v>Jalur ganda menghubungkan Cilegon Baru dan Cilegon Lama Sirkit 1.</v>
+        <v/>
       </c>
       <c r="W14" t="str">
         <v/>
@@ -1532,40 +1497,40 @@
         <v/>
       </c>
       <c r="C15" t="str">
-        <v>SUTT 150 kV CLBRU - CLGON Sirkit 2</v>
+        <v>Feeder Beban KTT SLFDO-1 (78 MVA)</v>
       </c>
       <c r="D15" t="str">
-        <v>Double Circuit Line 2</v>
+        <v>Feeder Beban</v>
       </c>
       <c r="E15" t="str">
-        <v>cb</v>
+        <v>Beban</v>
       </c>
       <c r="F15" t="str">
-        <v>CLBRU</v>
+        <v>SLRDA</v>
       </c>
       <c r="G15" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I15" t="str">
-        <v>CLGON</v>
+        <v>KTT SLFDO-1</v>
       </c>
       <c r="J15" t="str">
-        <v>busbar</v>
+        <v>Beban</v>
       </c>
       <c r="K15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L15" t="str">
-        <v>150 kV</v>
+        <v>20 kV</v>
       </c>
       <c r="M15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O15" t="str">
         <v>Beroperasi</v>
@@ -1574,13 +1539,13 @@
         <v>Normal</v>
       </c>
       <c r="Q15">
-        <v>50</v>
+        <v>78</v>
       </c>
       <c r="R15" t="str">
         <v/>
       </c>
       <c r="S15">
-        <v>11.2</v>
+        <v>1.2</v>
       </c>
       <c r="T15" t="str">
         <v>Banten - Cilegon</v>
@@ -1589,7 +1554,7 @@
         <v>JBB</v>
       </c>
       <c r="V15" t="str">
-        <v>Jalur ganda menghubungkan Cilegon Baru dan Cilegon Lama Sirkit 2.</v>
+        <v>Feeder Konsumen Industri KTT SLFDO-1</v>
       </c>
       <c r="W15" t="str">
         <v/>
@@ -1609,34 +1574,34 @@
         <v/>
       </c>
       <c r="C16" t="str">
-        <v>Bay Trafo Distribusi SRLYA</v>
+        <v>Feeder Beban KTT SLFDO-2 (30 MVA)</v>
       </c>
       <c r="D16" t="str">
-        <v>Bay Trafo</v>
+        <v>Feeder Beban</v>
       </c>
       <c r="E16" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="F16" t="str">
-        <v>SRLYA</v>
+        <v>SLRDA</v>
       </c>
       <c r="G16" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I16" t="str">
-        <v>Trafo Distribusi SRLYA</v>
+        <v>KTT SLFDO-2</v>
       </c>
       <c r="J16" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="K16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L16" t="str">
-        <v>150/20 kV</v>
+        <v>20 kV</v>
       </c>
       <c r="M16">
         <v>1</v>
@@ -1651,13 +1616,13 @@
         <v>Normal</v>
       </c>
       <c r="Q16">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="R16" t="str">
         <v/>
       </c>
       <c r="S16">
-        <v>0.1</v>
+        <v>1.2</v>
       </c>
       <c r="T16" t="str">
         <v>Banten - Cilegon</v>
@@ -1666,7 +1631,7 @@
         <v>JBB</v>
       </c>
       <c r="V16" t="str">
-        <v>Trafo pemakaian sendiri / distribusi lokal 150/20 kV Suralaya.</v>
+        <v>Feeder Konsumen Industri KTT SLFDO-2</v>
       </c>
       <c r="W16" t="str">
         <v/>
@@ -1686,34 +1651,34 @@
         <v/>
       </c>
       <c r="C17" t="str">
-        <v>Bay Trafo Distribusi CLBRU</v>
+        <v>Feeder Beban KTT PENDO (35 MVA)</v>
       </c>
       <c r="D17" t="str">
-        <v>Bay Trafo</v>
+        <v>Feeder Beban</v>
       </c>
       <c r="E17" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="F17" t="str">
-        <v>CLBRU</v>
+        <v>PENDO</v>
       </c>
       <c r="G17" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I17" t="str">
-        <v>Trafo Distribusi CLBRU</v>
+        <v>KTT PENDO</v>
       </c>
       <c r="J17" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="K17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L17" t="str">
-        <v>150/20 kV</v>
+        <v>20 kV</v>
       </c>
       <c r="M17">
         <v>1</v>
@@ -1728,13 +1693,13 @@
         <v>Normal</v>
       </c>
       <c r="Q17">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="R17" t="str">
         <v/>
       </c>
       <c r="S17">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="T17" t="str">
         <v>Banten - Cilegon</v>
@@ -1743,7 +1708,7 @@
         <v>JBB</v>
       </c>
       <c r="V17" t="str">
-        <v>Trafo distribusi lokal 150/20 kV Cilegon Baru.</v>
+        <v>Feeder Konsumen Industri KTT PENDO</v>
       </c>
       <c r="W17" t="str">
         <v/>
@@ -1760,37 +1725,37 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="C18" t="str">
-        <v>Feeder Trafo SLRDA ke KTT SLFDO-1</v>
+        <v>Feeder Beban KTT PENI (40 MVA)</v>
       </c>
       <c r="D18" t="str">
-        <v>Feeder KTT</v>
+        <v>Feeder Beban</v>
       </c>
       <c r="E18" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="F18" t="str">
-        <v>SLRDA</v>
+        <v>PENI</v>
       </c>
       <c r="G18" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H18">
         <v>2</v>
       </c>
       <c r="I18" t="str">
-        <v>KTT SLFDO-1</v>
+        <v>KTT PENI</v>
       </c>
       <c r="J18" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="K18">
         <v>3</v>
       </c>
       <c r="L18" t="str">
-        <v>150/20 kV</v>
+        <v>20 kV</v>
       </c>
       <c r="M18">
         <v>1</v>
@@ -1802,16 +1767,16 @@
         <v>Beroperasi</v>
       </c>
       <c r="P18" t="str">
-        <v>Normal</v>
+        <v>N-1</v>
       </c>
       <c r="Q18">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="R18" t="str">
         <v/>
       </c>
       <c r="S18">
-        <v>1.2</v>
+        <v>0.5</v>
       </c>
       <c r="T18" t="str">
         <v>Banten - Cilegon</v>
@@ -1820,7 +1785,7 @@
         <v>JBB</v>
       </c>
       <c r="V18" t="str">
-        <v>Suplai konsumen KTT SLFDO-1 Kapasitas 78 MVA</v>
+        <v>Feeder Konsumen Industri KTT PENI</v>
       </c>
       <c r="W18" t="str">
         <v/>
@@ -1840,37 +1805,37 @@
         <v/>
       </c>
       <c r="C19" t="str">
-        <v>Feeder Trafo SLRDA ke KTT SLFDO-2</v>
+        <v>Feeder Beban KTT LCI (115 MVA)</v>
       </c>
       <c r="D19" t="str">
-        <v>Feeder KTT</v>
+        <v>Feeder Beban</v>
       </c>
       <c r="E19" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="F19" t="str">
-        <v>SLRDA</v>
+        <v>PENI</v>
       </c>
       <c r="G19" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H19">
         <v>2</v>
       </c>
       <c r="I19" t="str">
-        <v>KTT SLFDO-2</v>
+        <v>KTT LCI</v>
       </c>
       <c r="J19" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="K19">
         <v>3</v>
       </c>
       <c r="L19" t="str">
-        <v>150/20 kV</v>
+        <v>20 kV</v>
       </c>
       <c r="M19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N19">
         <v>1</v>
@@ -1882,13 +1847,13 @@
         <v>Normal</v>
       </c>
       <c r="Q19">
-        <v>65</v>
-      </c>
-      <c r="R19" t="str">
-        <v/>
+        <v>58</v>
+      </c>
+      <c r="R19">
+        <v>57</v>
       </c>
       <c r="S19">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="T19" t="str">
         <v>Banten - Cilegon</v>
@@ -1897,7 +1862,7 @@
         <v>JBB</v>
       </c>
       <c r="V19" t="str">
-        <v>Suplai konsumen KTT SLFDO-2 Kapasitas 30 MVA</v>
+        <v>Feeder Konsumen Industri KTT LCI</v>
       </c>
       <c r="W19" t="str">
         <v/>
@@ -1917,34 +1882,34 @@
         <v/>
       </c>
       <c r="C20" t="str">
-        <v>Feeder Trafo PENDO ke KTT PENDO</v>
+        <v>Feeder Beban KTT MCCI (40 MVA)</v>
       </c>
       <c r="D20" t="str">
-        <v>Feeder KTT</v>
+        <v>Feeder Beban</v>
       </c>
       <c r="E20" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="F20" t="str">
-        <v>PENDO</v>
+        <v>MCCI5</v>
       </c>
       <c r="G20" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="H20">
         <v>2</v>
       </c>
       <c r="I20" t="str">
-        <v>KTT PENDO</v>
+        <v>KTT MCCI</v>
       </c>
       <c r="J20" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="K20">
         <v>3</v>
       </c>
       <c r="L20" t="str">
-        <v>150/20 kV</v>
+        <v>20 kV</v>
       </c>
       <c r="M20">
         <v>1</v>
@@ -1959,13 +1924,13 @@
         <v>Normal</v>
       </c>
       <c r="Q20">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="R20" t="str">
         <v/>
       </c>
       <c r="S20">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="T20" t="str">
         <v>Banten - Cilegon</v>
@@ -1974,7 +1939,7 @@
         <v>JBB</v>
       </c>
       <c r="V20" t="str">
-        <v>Suplai konsumen KTT PENDO Kapasitas 35 MVA</v>
+        <v>Feeder Konsumen Industri KTT MCCI</v>
       </c>
       <c r="W20" t="str">
         <v/>
@@ -1991,37 +1956,37 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v>Feeder Beban KTT MTSUI (31 MVA)</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Feeder Beban</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="F21" t="str">
+        <v>MTSUI</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Busbar</v>
+      </c>
+      <c r="H21">
         <v>3</v>
       </c>
-      <c r="C21" t="str">
-        <v>Feeder Trafo PENI ke KTT PENI</v>
-      </c>
-      <c r="D21" t="str">
-        <v>Feeder KTT</v>
-      </c>
-      <c r="E21" t="str">
-        <v>trafo_distribusi</v>
-      </c>
-      <c r="F21" t="str">
-        <v>PENI</v>
-      </c>
-      <c r="G21" t="str">
-        <v>busbar</v>
-      </c>
-      <c r="H21">
-        <v>2</v>
-      </c>
       <c r="I21" t="str">
-        <v>KTT PENI</v>
+        <v>KTT MTSUI</v>
       </c>
       <c r="J21" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="K21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L21" t="str">
-        <v>150/20 kV</v>
+        <v>20 kV</v>
       </c>
       <c r="M21">
         <v>1</v>
@@ -2033,16 +1998,16 @@
         <v>Beroperasi</v>
       </c>
       <c r="P21" t="str">
-        <v>N-1</v>
+        <v>Normal</v>
       </c>
       <c r="Q21">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="R21" t="str">
         <v/>
       </c>
       <c r="S21">
-        <v>1.1</v>
+        <v>0.4</v>
       </c>
       <c r="T21" t="str">
         <v>Banten - Cilegon</v>
@@ -2051,586 +2016,28 @@
         <v>JBB</v>
       </c>
       <c r="V21" t="str">
-        <v>Suplai konsumen KTT PENI Chandra Asri Kapasitas 40 MVA</v>
+        <v>Feeder Konsumen Industri KTT Mitsui</v>
       </c>
       <c r="W21" t="str">
-        <v>Terdapat risiko suplai saat pemeliharaan ruas single phi.</v>
+        <v/>
       </c>
       <c r="X21" t="str">
-        <v>Penyesuaian jadwal dengan konsumen industri.</v>
+        <v/>
       </c>
       <c r="Y21" t="str">
-        <v>Usulan double phi transmisi 150 kV.</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="str">
-        <v/>
-      </c>
-      <c r="C22" t="str">
-        <v>Feeder Trafo PENI ke KTT LCI</v>
-      </c>
-      <c r="D22" t="str">
-        <v>Feeder KTT</v>
-      </c>
-      <c r="E22" t="str">
-        <v>trafo_distribusi</v>
-      </c>
-      <c r="F22" t="str">
-        <v>PENI</v>
-      </c>
-      <c r="G22" t="str">
-        <v>busbar</v>
-      </c>
-      <c r="H22">
-        <v>2</v>
-      </c>
-      <c r="I22" t="str">
-        <v>KTT LCI</v>
-      </c>
-      <c r="J22" t="str">
-        <v>trafo_distribusi</v>
-      </c>
-      <c r="K22">
-        <v>3</v>
-      </c>
-      <c r="L22" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="M22">
-        <v>2</v>
-      </c>
-      <c r="N22">
-        <v>1</v>
-      </c>
-      <c r="O22" t="str">
-        <v>Beroperasi</v>
-      </c>
-      <c r="P22" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="Q22">
-        <v>64</v>
-      </c>
-      <c r="R22" t="str">
-        <v/>
-      </c>
-      <c r="S22">
-        <v>1.5</v>
-      </c>
-      <c r="T22" t="str">
-        <v>Banten - Cilegon</v>
-      </c>
-      <c r="U22" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="V22" t="str">
-        <v>Suplai 2 sirkit konsumen KTT LCI Kapasitas 115 MVA</v>
-      </c>
-      <c r="W22" t="str">
-        <v/>
-      </c>
-      <c r="X22" t="str">
-        <v/>
-      </c>
-      <c r="Y22" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="str">
-        <v/>
-      </c>
-      <c r="C23" t="str">
-        <v>Feeder Trafo MCCI5 ke KTT MCCI</v>
-      </c>
-      <c r="D23" t="str">
-        <v>Feeder KTT</v>
-      </c>
-      <c r="E23" t="str">
-        <v>trafo_distribusi</v>
-      </c>
-      <c r="F23" t="str">
-        <v>MCCI5</v>
-      </c>
-      <c r="G23" t="str">
-        <v>busbar</v>
-      </c>
-      <c r="H23">
-        <v>2</v>
-      </c>
-      <c r="I23" t="str">
-        <v>KTT MCCI</v>
-      </c>
-      <c r="J23" t="str">
-        <v>trafo_distribusi</v>
-      </c>
-      <c r="K23">
-        <v>3</v>
-      </c>
-      <c r="L23" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="M23">
-        <v>1</v>
-      </c>
-      <c r="N23">
-        <v>1</v>
-      </c>
-      <c r="O23" t="str">
-        <v>Beroperasi</v>
-      </c>
-      <c r="P23" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="Q23">
-        <v>55</v>
-      </c>
-      <c r="R23" t="str">
-        <v/>
-      </c>
-      <c r="S23">
-        <v>0.9</v>
-      </c>
-      <c r="T23" t="str">
-        <v>Banten - Cilegon</v>
-      </c>
-      <c r="U23" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="V23" t="str">
-        <v>Suplai konsumen KTT MCCI Kapasitas 40 MVA</v>
-      </c>
-      <c r="W23" t="str">
-        <v/>
-      </c>
-      <c r="X23" t="str">
-        <v/>
-      </c>
-      <c r="Y23" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" t="str">
-        <v/>
-      </c>
-      <c r="C24" t="str">
-        <v>Bay Trafo Distribusi CLGON</v>
-      </c>
-      <c r="D24" t="str">
-        <v>Bay Trafo</v>
-      </c>
-      <c r="E24" t="str">
-        <v>trafo_distribusi</v>
-      </c>
-      <c r="F24" t="str">
-        <v>CLGON</v>
-      </c>
-      <c r="G24" t="str">
-        <v>busbar</v>
-      </c>
-      <c r="H24">
-        <v>2</v>
-      </c>
-      <c r="I24" t="str">
-        <v>Trafo Distribusi CLGON</v>
-      </c>
-      <c r="J24" t="str">
-        <v>trafo_distribusi</v>
-      </c>
-      <c r="K24">
-        <v>3</v>
-      </c>
-      <c r="L24" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="M24">
-        <v>1</v>
-      </c>
-      <c r="N24">
-        <v>1</v>
-      </c>
-      <c r="O24" t="str">
-        <v>Beroperasi</v>
-      </c>
-      <c r="P24" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="Q24">
-        <v>52</v>
-      </c>
-      <c r="R24" t="str">
-        <v/>
-      </c>
-      <c r="S24">
-        <v>0.1</v>
-      </c>
-      <c r="T24" t="str">
-        <v>Banten - Cilegon</v>
-      </c>
-      <c r="U24" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="V24" t="str">
-        <v>Trafo distribusi lokal 150/20 kV Cilegon Lama.</v>
-      </c>
-      <c r="W24" t="str">
-        <v/>
-      </c>
-      <c r="X24" t="str">
-        <v/>
-      </c>
-      <c r="Y24" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="str">
-        <v/>
-      </c>
-      <c r="C25" t="str">
-        <v>Feeder Trafo MTSUI ke KTT MTSUI</v>
-      </c>
-      <c r="D25" t="str">
-        <v>Feeder KTT</v>
-      </c>
-      <c r="E25" t="str">
-        <v>trafo_distribusi</v>
-      </c>
-      <c r="F25" t="str">
-        <v>MTSUI</v>
-      </c>
-      <c r="G25" t="str">
-        <v>busbar</v>
-      </c>
-      <c r="H25">
-        <v>3</v>
-      </c>
-      <c r="I25" t="str">
-        <v>KTT MTSUI</v>
-      </c>
-      <c r="J25" t="str">
-        <v>trafo_distribusi</v>
-      </c>
-      <c r="K25">
-        <v>4</v>
-      </c>
-      <c r="L25" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="M25">
-        <v>1</v>
-      </c>
-      <c r="N25">
-        <v>1</v>
-      </c>
-      <c r="O25" t="str">
-        <v>Beroperasi</v>
-      </c>
-      <c r="P25" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="Q25">
-        <v>50</v>
-      </c>
-      <c r="R25" t="str">
-        <v/>
-      </c>
-      <c r="S25">
-        <v>0.7</v>
-      </c>
-      <c r="T25" t="str">
-        <v>Banten - Cilegon</v>
-      </c>
-      <c r="U25" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="V25" t="str">
-        <v>Suplai konsumen KTT MTSUI Kapasitas 31 MVA</v>
-      </c>
-      <c r="W25" t="str">
-        <v/>
-      </c>
-      <c r="X25" t="str">
-        <v/>
-      </c>
-      <c r="Y25" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="str">
-        <v/>
-      </c>
-      <c r="C26" t="str">
-        <v>Bay Feeder CLBRU ke KSTEL (Rencana)</v>
-      </c>
-      <c r="D26" t="str">
-        <v>Bay Rencana</v>
-      </c>
-      <c r="E26" t="str">
-        <v>cb</v>
-      </c>
-      <c r="F26" t="str">
-        <v>CLBRU</v>
-      </c>
-      <c r="G26" t="str">
-        <v>busbar</v>
-      </c>
-      <c r="H26">
-        <v>1</v>
-      </c>
-      <c r="I26" t="str">
-        <v>KSTEL</v>
-      </c>
-      <c r="J26" t="str">
-        <v>cb</v>
-      </c>
-      <c r="K26">
-        <v>3</v>
-      </c>
-      <c r="L26" t="str">
-        <v>150 kV</v>
-      </c>
-      <c r="M26">
-        <v>1</v>
-      </c>
-      <c r="N26">
-        <v>1</v>
-      </c>
-      <c r="O26" t="str">
-        <v>Rencana</v>
-      </c>
-      <c r="P26" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="Q26">
-        <v>0</v>
-      </c>
-      <c r="R26" t="str">
-        <v/>
-      </c>
-      <c r="S26">
-        <v>3.5</v>
-      </c>
-      <c r="T26" t="str">
-        <v>Banten - Cilegon</v>
-      </c>
-      <c r="U26" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="V26" t="str">
-        <v>Bay Rencana Penghantar KSTEL (Dashed Line)</v>
-      </c>
-      <c r="W26" t="str">
-        <v/>
-      </c>
-      <c r="X26" t="str">
-        <v/>
-      </c>
-      <c r="Y26" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="str">
-        <v/>
-      </c>
-      <c r="C27" t="str">
-        <v>Bay Feeder CLBRU ke POSCO (Rencana)</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Bay Rencana</v>
-      </c>
-      <c r="E27" t="str">
-        <v>cb</v>
-      </c>
-      <c r="F27" t="str">
-        <v>CLBRU</v>
-      </c>
-      <c r="G27" t="str">
-        <v>busbar</v>
-      </c>
-      <c r="H27">
-        <v>1</v>
-      </c>
-      <c r="I27" t="str">
-        <v>POSCO</v>
-      </c>
-      <c r="J27" t="str">
-        <v>cb</v>
-      </c>
-      <c r="K27">
-        <v>3</v>
-      </c>
-      <c r="L27" t="str">
-        <v>150 kV</v>
-      </c>
-      <c r="M27">
-        <v>1</v>
-      </c>
-      <c r="N27">
-        <v>1</v>
-      </c>
-      <c r="O27" t="str">
-        <v>Rencana</v>
-      </c>
-      <c r="P27" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="Q27">
-        <v>0</v>
-      </c>
-      <c r="R27" t="str">
-        <v/>
-      </c>
-      <c r="S27">
-        <v>4.2</v>
-      </c>
-      <c r="T27" t="str">
-        <v>Banten - Cilegon</v>
-      </c>
-      <c r="U27" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="V27" t="str">
-        <v>Bay Rencana Penghantar POSCO (Dashed Line)</v>
-      </c>
-      <c r="W27" t="str">
-        <v/>
-      </c>
-      <c r="X27" t="str">
-        <v/>
-      </c>
-      <c r="Y27" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" t="str">
-        <v/>
-      </c>
-      <c r="C28" t="str">
-        <v>Bay Feeder CLGON ke KSTEL (Rencana)</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Bay Rencana</v>
-      </c>
-      <c r="E28" t="str">
-        <v>cb</v>
-      </c>
-      <c r="F28" t="str">
-        <v>CLGON</v>
-      </c>
-      <c r="G28" t="str">
-        <v>busbar</v>
-      </c>
-      <c r="H28">
-        <v>2</v>
-      </c>
-      <c r="I28" t="str">
-        <v>KSTEL</v>
-      </c>
-      <c r="J28" t="str">
-        <v>cb</v>
-      </c>
-      <c r="K28">
-        <v>3</v>
-      </c>
-      <c r="L28" t="str">
-        <v>150 kV</v>
-      </c>
-      <c r="M28">
-        <v>1</v>
-      </c>
-      <c r="N28">
-        <v>1</v>
-      </c>
-      <c r="O28" t="str">
-        <v>Rencana</v>
-      </c>
-      <c r="P28" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="Q28">
-        <v>0</v>
-      </c>
-      <c r="R28" t="str">
-        <v/>
-      </c>
-      <c r="S28">
-        <v>2.8</v>
-      </c>
-      <c r="T28" t="str">
-        <v>Banten - Cilegon</v>
-      </c>
-      <c r="U28" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="V28" t="str">
-        <v>Bay Rencana Penghantar KSTEL dari CLGON (Dashed Line)</v>
-      </c>
-      <c r="W28" t="str">
-        <v/>
-      </c>
-      <c r="X28" t="str">
-        <v/>
-      </c>
-      <c r="Y28" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Y28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q28"/>
-  <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="16.83203125" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" customWidth="1"/>
-    <col min="14" max="14" width="45.83203125" customWidth="1"/>
-    <col min="15" max="15" width="35.83203125" customWidth="1"/>
-    <col min="16" max="16" width="35.83203125" customWidth="1"/>
-    <col min="17" max="17" width="35.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:Q25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2696,10 +2103,10 @@
         <v>Suralaya Baru</v>
       </c>
       <c r="D2" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E2" t="str">
-        <v>Panjang (Wide Busbar)</v>
+        <v>Normal</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -2726,7 +2133,7 @@
         <v>JBB</v>
       </c>
       <c r="N2" t="str">
-        <v>Rel Busbar 500 kV Suralaya Baru (Warna Biru)</v>
+        <v>Busbar 500 kV Suralaya Baru</v>
       </c>
       <c r="O2" t="str">
         <v/>
@@ -2749,10 +2156,10 @@
         <v>Suralaya</v>
       </c>
       <c r="D3" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E3" t="str">
-        <v>Panjang (Wide Busbar)</v>
+        <v>Normal</v>
       </c>
       <c r="F3" t="str">
         <v/>
@@ -2779,7 +2186,7 @@
         <v>JBB</v>
       </c>
       <c r="N3" t="str">
-        <v>Rel Busbar 500 kV Suralaya (Warna Biru)</v>
+        <v>Busbar 500 kV Suralaya</v>
       </c>
       <c r="O3" t="str">
         <v/>
@@ -2802,10 +2209,10 @@
         <v>Cilegon Baru</v>
       </c>
       <c r="D4" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E4" t="str">
-        <v>Panjang (Wide Busbar)</v>
+        <v>Normal</v>
       </c>
       <c r="F4" t="str">
         <v/>
@@ -2832,7 +2239,7 @@
         <v>JBB</v>
       </c>
       <c r="N4" t="str">
-        <v>Rel Busbar 500 kV Cilegon Baru (Warna Biru)</v>
+        <v>Busbar 500 kV Cilegon Baru</v>
       </c>
       <c r="O4" t="str">
         <v/>
@@ -2855,7 +2262,7 @@
         <v>Unit 3</v>
       </c>
       <c r="D5" t="str">
-        <v>generator</v>
+        <v>Pembangkit</v>
       </c>
       <c r="E5" t="str">
         <v>Normal</v>
@@ -2885,7 +2292,7 @@
         <v>JBB</v>
       </c>
       <c r="N5" t="str">
-        <v>Generator Pembangkit Unit 3 (Lingkaran Hijau + Simbol AC ~) dengan Step-up GSUT</v>
+        <v>Bay Pembangkit: 1. Pembangkit, 2. Trafo Generator, 3. CB</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -2897,7 +2304,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" xml:space="preserve">
+    <row r="6">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2908,7 +2315,7 @@
         <v>IBT 2 SRL-BARU</v>
       </c>
       <c r="D6" t="str">
-        <v>ibt</v>
+        <v>IBT</v>
       </c>
       <c r="E6" t="str">
         <v>Normal</v>
@@ -2938,24 +2345,19 @@
         <v>JBB</v>
       </c>
       <c r="N6" t="str">
-        <v>Pembebanan IBT–1,2 Suralaya tidak memenuhi kriteria N–1 saat PLTU Suralaya unit–3 tidak beroperasi dan IBT–4 Cilegon masuk sub sistem Cilegon.</v>
-      </c>
-      <c r="O6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Pemeliharaan IBT sulit dilakukan.
-2. Pertumbuhan beban menjadi terhambat.
-3. Terjadi pemadaman apabila trip salah satu IBT di Suralaya.</v>
-      </c>
-      <c r="P6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW.
-2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan target total 137 MW.
-3. Pemeliharaan IBT saat beban rendah.</v>
-      </c>
-      <c r="Q6" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. COD Tahun 2025.</v>
-      </c>
-    </row>
-    <row r="7" xml:space="preserve">
+        <v>Pembebanan IBT–1,2 Suralaya tidak memenuhi kriteria N–1 saat PLTU Suralaya unit–3 tidak beroperasi.</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Pemadaman apabila trip salah satu IBT.</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Terpasang DS OLS IBT 1,2 Suralaya.</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>Uprating IBT–1 &amp; 2 dari 250 MVA menjadi 500 MVA.</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2966,7 +2368,7 @@
         <v>IBT 1 SRLYA</v>
       </c>
       <c r="D7" t="str">
-        <v>ibt</v>
+        <v>IBT</v>
       </c>
       <c r="E7" t="str">
         <v>Normal</v>
@@ -2996,22 +2398,19 @@
         <v>JBB</v>
       </c>
       <c r="N7" t="str">
-        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA sedangkan IBT #4 Cilegon 500 MVA).</v>
-      </c>
-      <c r="O7" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Ketidakseimbangan beban antara IBT Suralaya dan IBT Cilegon.
-2. Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
-      </c>
-      <c r="P7" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya.
-2. Pemeliharaan IBT saat beban rendah.</v>
-      </c>
-      <c r="Q7" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. COD Tahun 2026.</v>
-      </c>
-    </row>
-    <row r="8" xml:space="preserve">
+        <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA).</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Overload pada IBT Suralaya.</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Terpasang DS OLS IBT 1,2 Suralaya.</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>Uprating IBT–1 &amp; 2 dari 250 MVA menjadi 500 MVA.</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3022,7 +2421,7 @@
         <v>IBT 4 CLBRU</v>
       </c>
       <c r="D8" t="str">
-        <v>ibt</v>
+        <v>IBT</v>
       </c>
       <c r="E8" t="str">
         <v>Normal</v>
@@ -3055,14 +2454,13 @@
         <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #4 Cilegon 500 MVA).</v>
       </c>
       <c r="O8" t="str">
-        <v>Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
+        <v>Ketidakseimbangan beban.</v>
       </c>
       <c r="P8" t="str">
-        <v>Optimalisasi transfer trip dan defense scheme antar GI.</v>
-      </c>
-      <c r="Q8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya menjadi 500 MVA.</v>
+        <v>Optimalisasi transfer trip antar GI.</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Uprating IBT–1 &amp; 2 Suralaya menjadi 500 MVA.</v>
       </c>
     </row>
     <row r="9">
@@ -3070,13 +2468,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>Gardu Induk SRLYA (150 kV)</v>
+        <v>GI Suralaya 150 kV (Rel Busbar)</v>
       </c>
       <c r="C9" t="str">
         <v>SRLYA</v>
       </c>
       <c r="D9" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E9" t="str">
         <v>Panjang (Wide Busbar)</v>
@@ -3106,7 +2504,7 @@
         <v>JBB</v>
       </c>
       <c r="N9" t="str">
-        <v>Busbar Utama 150 kV Suralaya (Tier 1, Merah Panjang menampung Unit 3, IBT 1, IBT 2, dan 5 Saluran ke Bawah)</v>
+        <v>Busbar 150 kV Suralaya (Menghubungkan IBT 1, IBT 2, dan Saluran Distribusi)</v>
       </c>
       <c r="O9" t="str">
         <v/>
@@ -3123,13 +2521,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>Gardu Induk CLBRU (150 kV)</v>
+        <v>GI Cilegon Baru 150 kV (Rel Busbar)</v>
       </c>
       <c r="C10" t="str">
         <v>CLBRU</v>
       </c>
       <c r="D10" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E10" t="str">
         <v>Panjang (Wide Busbar)</v>
@@ -3159,7 +2557,7 @@
         <v>JBB</v>
       </c>
       <c r="N10" t="str">
-        <v>Busbar Utama 150 kV Cilegon Baru (Tier 1, Merah Panjang menghubungkan IBT 4 ke CLGON, Trafo Lokal, KSTEL, POSCO)</v>
+        <v>Busbar 150 kV Cilegon Baru</v>
       </c>
       <c r="O10" t="str">
         <v/>
@@ -3176,13 +2574,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>Gardu Induk SLRDA (150 kV)</v>
+        <v>GI Salira Indah</v>
       </c>
       <c r="C11" t="str">
         <v>SLRDA</v>
       </c>
       <c r="D11" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E11" t="str">
         <v>Normal</v>
@@ -3212,7 +2610,7 @@
         <v>JBB</v>
       </c>
       <c r="N11" t="str">
-        <v>Gardu Induk Salira Indah (Tier 2, Menyuplai KTT SLFDO-1 &amp; SLFDO-2)</v>
+        <v>Gardu Induk Salira Indah</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -3229,13 +2627,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>Gardu Induk PENDO (150 kV)</v>
+        <v>GI Pendo</v>
       </c>
       <c r="C12" t="str">
         <v>PENDO</v>
       </c>
       <c r="D12" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E12" t="str">
         <v>Normal</v>
@@ -3265,7 +2663,7 @@
         <v>JBB</v>
       </c>
       <c r="N12" t="str">
-        <v>Gardu Induk Pendo (Tier 2, Menyuplai KTT PENDO 35 MVA)</v>
+        <v>Gardu Induk Pendo</v>
       </c>
       <c r="O12" t="str">
         <v/>
@@ -3282,13 +2680,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>Gardu Induk PENI (150 kV)</v>
+        <v>GI Chandra Asri (PENI)</v>
       </c>
       <c r="C13" t="str">
         <v>PENI</v>
       </c>
       <c r="D13" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E13" t="str">
         <v>Normal</v>
@@ -3318,16 +2716,16 @@
         <v>JBB</v>
       </c>
       <c r="N13" t="str">
-        <v>Ruas Penghantar Suralaya–PENI–Mitsui–Cilegon masih single phi.</v>
+        <v>Ruas Penghantar Suralaya-PENI masih single phi.</v>
       </c>
       <c r="O13" t="str">
-        <v>Pemadaman apabila terdapat gangguan N–1–1.</v>
+        <v>Pemadaman apabila terdapat gangguan N-1-1.</v>
       </c>
       <c r="P13" t="str">
-        <v>Pemeliharaan mengikuti jadwal KTT industri.</v>
+        <v>Pemeliharaan mengikuti jadwal KTT.</v>
       </c>
       <c r="Q13" t="str">
-        <v>Double phi transmisi 150 kV COD 2030.</v>
+        <v>Double phi COD 2030.</v>
       </c>
     </row>
     <row r="14">
@@ -3335,13 +2733,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>Gardu Induk MCCI5 (150 kV)</v>
+        <v>GI Mitsubishi Chemical (MCCI)</v>
       </c>
       <c r="C14" t="str">
         <v>MCCI5</v>
       </c>
       <c r="D14" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E14" t="str">
         <v>Normal</v>
@@ -3371,13 +2769,13 @@
         <v>JBB</v>
       </c>
       <c r="N14" t="str">
-        <v>Ruas Penghantar Suralaya–MCCI–Cilegon masih single phi.</v>
+        <v>Ruas Penghantar Suralaya-MCCI-Cilegon masih single phi.</v>
       </c>
       <c r="O14" t="str">
-        <v>Pemadaman apabila trip saat pemeliharaan KTT.</v>
+        <v>Pemadaman apabila gangguan.</v>
       </c>
       <c r="P14" t="str">
-        <v>Penyesuaian jadwal pemeliharaan dari KTT.</v>
+        <v>Penyesuaian jadwal pemeliharaan.</v>
       </c>
       <c r="Q14" t="str">
         <v>Usulan double phi ruas Suralaya s.d Cilegon Lama.</v>
@@ -3388,13 +2786,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>Gardu Induk CLGON (150 kV)</v>
+        <v>GI Cilegon Lama</v>
       </c>
       <c r="C15" t="str">
         <v>CLGON</v>
       </c>
       <c r="D15" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E15" t="str">
         <v>Normal</v>
@@ -3424,7 +2822,7 @@
         <v>JBB</v>
       </c>
       <c r="N15" t="str">
-        <v>Gardu Induk Cilegon Lama (Menerima double circuit dari CLBRU, serta loop dari MCCI5 dan MTSUI)</v>
+        <v>Gardu Induk Cilegon Lama</v>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -3441,13 +2839,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>Gardu Induk MTSUI (150 kV)</v>
+        <v>GI Mitsui (MTSUI)</v>
       </c>
       <c r="C16" t="str">
         <v>MTSUI</v>
       </c>
       <c r="D16" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="E16" t="str">
         <v>Normal</v>
@@ -3477,16 +2875,16 @@
         <v>JBB</v>
       </c>
       <c r="N16" t="str">
-        <v>Ruas Peni–Mitsui–Cilegon masih single phi (Tier 3).</v>
+        <v>Ruas Mitsui-Cilegon single phi</v>
       </c>
       <c r="O16" t="str">
-        <v>Terjadi pemadaman apabila trip N-1.</v>
+        <v/>
       </c>
       <c r="P16" t="str">
-        <v>Pengaturan konfigurasi jaringan.</v>
+        <v/>
       </c>
       <c r="Q16" t="str">
-        <v>Double phi ruas Suralaya s.d Cilegon Lama.</v>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -3494,13 +2892,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>KTT SLFDO-1</v>
+        <v>Konsumen KTT SLFDO-1 (78 MVA)</v>
       </c>
       <c r="C17" t="str">
         <v>KTT SLFDO-1</v>
       </c>
       <c r="D17" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="E17" t="str">
         <v>Normal</v>
@@ -3530,7 +2928,7 @@
         <v>JBB</v>
       </c>
       <c r="N17" t="str">
-        <v>Konsumen Tegangan Tinggi SLFDO-1 (78 MVA)</v>
+        <v>Konsumen Tegangan Tinggi SLFDO-1</v>
       </c>
       <c r="O17" t="str">
         <v/>
@@ -3547,13 +2945,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>KTT SLFDO-2</v>
+        <v>Konsumen KTT SLFDO-2 (30 MVA)</v>
       </c>
       <c r="C18" t="str">
         <v>KTT SLFDO-2</v>
       </c>
       <c r="D18" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="E18" t="str">
         <v>Normal</v>
@@ -3583,7 +2981,7 @@
         <v>JBB</v>
       </c>
       <c r="N18" t="str">
-        <v>Konsumen Tegangan Tinggi SLFDO-2 (30 MVA)</v>
+        <v>Konsumen Tegangan Tinggi SLFDO-2</v>
       </c>
       <c r="O18" t="str">
         <v/>
@@ -3600,13 +2998,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>KTT PENDO</v>
+        <v>Konsumen KTT PENDO (35 MVA)</v>
       </c>
       <c r="C19" t="str">
         <v>KTT PENDO</v>
       </c>
       <c r="D19" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="E19" t="str">
         <v>Normal</v>
@@ -3636,7 +3034,7 @@
         <v>JBB</v>
       </c>
       <c r="N19" t="str">
-        <v>Konsumen Tegangan Tinggi PENDO (35 MVA)</v>
+        <v>Konsumen Tegangan Tinggi PENDO</v>
       </c>
       <c r="O19" t="str">
         <v/>
@@ -3653,13 +3051,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>KTT PENI</v>
+        <v>Konsumen KTT PENI (40 MVA)</v>
       </c>
       <c r="C20" t="str">
         <v>KTT PENI</v>
       </c>
       <c r="D20" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="E20" t="str">
         <v>Normal</v>
@@ -3689,16 +3087,16 @@
         <v>JBB</v>
       </c>
       <c r="N20" t="str">
-        <v>Konsumen Tegangan Tinggi PENI Chandra Asri (40 MVA, Memiliki Kerawanan #3)</v>
+        <v>Konsumen Tegangan Tinggi PENI Chandra Asri</v>
       </c>
       <c r="O20" t="str">
-        <v>Potensi kendala operasional saat gangguan ruas single phi.</v>
+        <v/>
       </c>
       <c r="P20" t="str">
-        <v>Jadwal pemeliharaan selaras dengan turn-around pabrik.</v>
+        <v/>
       </c>
       <c r="Q20" t="str">
-        <v>Usulan perkuatan sistem suplai transmisi.</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -3706,13 +3104,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>KTT LCI</v>
+        <v>Konsumen KTT LCI (115 MVA)</v>
       </c>
       <c r="C21" t="str">
         <v>KTT LCI</v>
       </c>
       <c r="D21" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="E21" t="str">
         <v>Normal</v>
@@ -3742,7 +3140,7 @@
         <v>JBB</v>
       </c>
       <c r="N21" t="str">
-        <v>Konsumen KTT LCI (115 MVA, Disuplai 2 Sirkit dengan 2 PMT CB)</v>
+        <v>Konsumen KTT LCI</v>
       </c>
       <c r="O21" t="str">
         <v/>
@@ -3759,13 +3157,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>KTT MCCI</v>
+        <v>Konsumen KTT MCCI (40 MVA)</v>
       </c>
       <c r="C22" t="str">
         <v>KTT MCCI</v>
       </c>
       <c r="D22" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="E22" t="str">
         <v>Normal</v>
@@ -3795,7 +3193,7 @@
         <v>JBB</v>
       </c>
       <c r="N22" t="str">
-        <v>Konsumen Tegangan Tinggi MCCI (40 MVA)</v>
+        <v>Konsumen KTT MCCI</v>
       </c>
       <c r="O22" t="str">
         <v/>
@@ -3812,13 +3210,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>KTT MTSUI</v>
+        <v>Konsumen KTT MTSUI (31 MVA)</v>
       </c>
       <c r="C23" t="str">
         <v>KTT MTSUI</v>
       </c>
       <c r="D23" t="str">
-        <v>trafo_distribusi</v>
+        <v>Beban</v>
       </c>
       <c r="E23" t="str">
         <v>Normal</v>
@@ -3848,7 +3246,7 @@
         <v>JBB</v>
       </c>
       <c r="N23" t="str">
-        <v>Konsumen Tegangan Tinggi Mitsui (31 MVA, Terhubung ke GI MTSUI)</v>
+        <v>Konsumen KTT Mitsui</v>
       </c>
       <c r="O23" t="str">
         <v/>
@@ -3865,25 +3263,25 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>Trafo Distribusi SRLYA</v>
+        <v>Konsumen KSTEL (Krakatau Steel)</v>
       </c>
       <c r="C24" t="str">
-        <v>Trafo SRLYA</v>
+        <v>KSTEL</v>
       </c>
       <c r="D24" t="str">
-        <v>trafo_distribusi</v>
+        <v>Busbar</v>
       </c>
       <c r="E24" t="str">
         <v>Normal</v>
       </c>
       <c r="F24" t="str">
-        <v>60 MVA</v>
+        <v/>
       </c>
       <c r="G24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H24" t="str">
-        <v>150/20 kV</v>
+        <v>150 kV</v>
       </c>
       <c r="I24" t="str">
         <v/>
@@ -3901,7 +3299,7 @@
         <v>JBB</v>
       </c>
       <c r="N24" t="str">
-        <v>Trafo distribusi lokal 150/20 kV Suralaya</v>
+        <v>Konsumen KSTEL (Krakatau Steel)</v>
       </c>
       <c r="O24" t="str">
         <v/>
@@ -3918,25 +3316,25 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>Trafo Distribusi CLBRU</v>
+        <v>Konsumen POSCO (Krakatau POSCO)</v>
       </c>
       <c r="C25" t="str">
-        <v>Trafo CLBRU</v>
+        <v>POSCO</v>
       </c>
       <c r="D25" t="str">
-        <v>trafo_distribusi</v>
+        <v>Busbar</v>
       </c>
       <c r="E25" t="str">
         <v>Normal</v>
       </c>
       <c r="F25" t="str">
-        <v>60 MVA</v>
+        <v/>
       </c>
       <c r="G25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H25" t="str">
-        <v>150/20 kV</v>
+        <v>150 kV</v>
       </c>
       <c r="I25" t="str">
         <v/>
@@ -3954,7 +3352,7 @@
         <v>JBB</v>
       </c>
       <c r="N25" t="str">
-        <v>Trafo distribusi lokal 150/20 kV Cilegon Baru</v>
+        <v>Konsumen Krakatau POSCO</v>
       </c>
       <c r="O25" t="str">
         <v/>
@@ -3963,185 +3361,19 @@
         <v/>
       </c>
       <c r="Q25" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="str">
-        <v>Trafo Distribusi CLGON</v>
-      </c>
-      <c r="C26" t="str">
-        <v>Trafo CLGON</v>
-      </c>
-      <c r="D26" t="str">
-        <v>trafo_distribusi</v>
-      </c>
-      <c r="E26" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="F26" t="str">
-        <v>60 MVA</v>
-      </c>
-      <c r="G26">
-        <v>3</v>
-      </c>
-      <c r="H26" t="str">
-        <v>150/20 kV</v>
-      </c>
-      <c r="I26" t="str">
-        <v/>
-      </c>
-      <c r="J26" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="K26" t="str">
-        <v/>
-      </c>
-      <c r="L26" t="str">
-        <v>Banten</v>
-      </c>
-      <c r="M26" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="N26" t="str">
-        <v>Trafo distribusi lokal 150/20 kV Cilegon Lama</v>
-      </c>
-      <c r="O26" t="str">
-        <v/>
-      </c>
-      <c r="P26" t="str">
-        <v/>
-      </c>
-      <c r="Q26" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="str">
-        <v>KSTEL</v>
-      </c>
-      <c r="C27" t="str">
-        <v>KSTEL</v>
-      </c>
-      <c r="D27" t="str">
-        <v>cb</v>
-      </c>
-      <c r="E27" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="F27" t="str">
-        <v/>
-      </c>
-      <c r="G27">
-        <v>3</v>
-      </c>
-      <c r="H27" t="str">
-        <v>150 kV</v>
-      </c>
-      <c r="I27" t="str">
-        <v/>
-      </c>
-      <c r="J27" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="K27" t="str">
-        <v/>
-      </c>
-      <c r="L27" t="str">
-        <v>Banten</v>
-      </c>
-      <c r="M27" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="N27" t="str">
-        <v>Bay Rencana Konsumen Krakatau Steel (KSTEL) Garis Putus-putus</v>
-      </c>
-      <c r="O27" t="str">
-        <v/>
-      </c>
-      <c r="P27" t="str">
-        <v/>
-      </c>
-      <c r="Q27" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" t="str">
-        <v>POSCO</v>
-      </c>
-      <c r="C28" t="str">
-        <v>POSCO</v>
-      </c>
-      <c r="D28" t="str">
-        <v>cb</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="F28" t="str">
-        <v/>
-      </c>
-      <c r="G28">
-        <v>3</v>
-      </c>
-      <c r="H28" t="str">
-        <v>150 kV</v>
-      </c>
-      <c r="I28" t="str">
-        <v/>
-      </c>
-      <c r="J28" t="str">
-        <v>Normal</v>
-      </c>
-      <c r="K28" t="str">
-        <v/>
-      </c>
-      <c r="L28" t="str">
-        <v>Banten</v>
-      </c>
-      <c r="M28" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="N28" t="str">
-        <v>Bay Rencana Konsumen Krakatau Posco (POSCO) Garis Putus-putus</v>
-      </c>
-      <c r="O28" t="str">
-        <v/>
-      </c>
-      <c r="P28" t="str">
-        <v/>
-      </c>
-      <c r="Q28" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q25"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
-  <cols>
-    <col min="1" max="1" width="26.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="48.83203125" customWidth="1"/>
-    <col min="4" max="4" width="55.83203125" customWidth="1"/>
-    <col min="5" max="5" width="45.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:E9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4162,127 +3394,150 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>1. Pembangkit / Generator</v>
+        <v>Peralatan (1)</v>
       </c>
       <c r="B2" t="str">
-        <v>generator</v>
+        <v>Generator / Pembangkit</v>
       </c>
       <c r="C2" t="str">
-        <v>Lingkaran Hijau + Simbol Gelombang AC (~)</v>
+        <v>Lingkaran Hijau dengan Gelombang Sinus AC (~)</v>
       </c>
       <c r="D2" t="str">
-        <v>Digunakan untuk merepresentasikan sumber daya pembangkitan (PLTU, PLTGU, PLTA, dll). Pada diagram terletak di bagian paling atas (Unit 3).</v>
+        <v>Titik hulu pembangkit listrik utama (PLTU, PLTA, PLTG, PLTGU).</v>
       </c>
       <c r="E2" t="str">
-        <v>PLTU Suralaya Unit 3, PLTGU Muara Karang Unit 1-3</v>
+        <v>PLTU Suralaya Unit 3 (600 MW)</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2. Trafo Generator (GSUT)</v>
+        <v>Peralatan (2)</v>
       </c>
       <c r="B3" t="str">
-        <v>trafo_generator</v>
+        <v>Trafo Generator (GSUT)</v>
       </c>
       <c r="C3" t="str">
-        <v>Dua Cincin Bertaut: Atas Hijau (Generator), Bawah Merah (Tegangan Tinggi)</v>
+        <v>2 Lingkaran Interlocking (Atas: Hijau sisi Gen, Bawah: Merah sisi GI)</v>
       </c>
       <c r="D3" t="str">
-        <v>Digunakan untuk menaikkan tegangan dari generator pembangkit ke tegangan sistem transmisi (Generator Step-Up Transformer / GSUT).</v>
+        <v>Trafo penaik tegangan generator (Generator Step-Up) dari 15-20 kV ke tegangan tinggi GI (150/500 kV).</v>
       </c>
       <c r="E3" t="str">
-        <v>Trafo Step-Up PLTU Unit 3 ke Busbar 150 kV SRLYA</v>
+        <v>Bay Pembangkit ke Busbar GI</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>3. Circuit Breaker (PMT)</v>
+        <v>Switching (3)</v>
       </c>
       <c r="B4" t="str">
-        <v>cb</v>
+        <v>CB / PMT (Pemutus Tenaga)</v>
       </c>
       <c r="C4" t="str">
-        <v>Balok Persegi Merah Solid pada Jalur Penghantar</v>
+        <v>Balok / Persegi Panjang Solid Merah Tegak dengan garis terminal</v>
       </c>
       <c r="D4" t="str">
-        <v>Pemutus Tenaga (PMT / Circuit Breaker) yang diletakkan pada bay pengirim maupun penerima GI ke GI untuk memutus arus gangguan.</v>
+        <v>Circuit Breaker pada bay pengirim dan penerima GI ke GI untuk memutus beban dan gangguan arus pendek.</v>
       </c>
       <c r="E4" t="str">
-        <v>Semua bay outgoing/incoming SUTT 150 kV, bay trafo, dan bay IBT</v>
+        <v>Bay Line, Bay IBT, Bay Trafo, Bay Generator</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>4. Interbus Transformer (IBT)</v>
+        <v>Peralatan (4)</v>
       </c>
       <c r="B5" t="str">
-        <v>ibt</v>
+        <v>IBT (Interbus Transformer)</v>
       </c>
       <c r="C5" t="str">
-        <v>Tiga Cincin Bertaut: Atas Biru (500 kV), Kiri Merah (150 kV), Kanan Kuning (Tertiary 33/20 kV)</v>
+        <v>3 Lingkaran Bertumpuk (Atas Biru 500kV, Kiri Merah 150kV, Kanan Kuning 33kV)</v>
       </c>
       <c r="D5" t="str">
-        <v>Transformator Daya Besar (3 Winding) penghubung antar grid tegangan ekstra tinggi 500 kV atau 275 kV ke tegangan transmisi 150 kV.</v>
+        <v>Trafo interkoneksi sistem transmisi tegangan ekstra tinggi (500/150 kV atau 275/150 kV).</v>
       </c>
       <c r="E5" t="str">
-        <v>IBT 1 Suralaya (500/150 kV), IBT 2 Suralaya Baru, IBT 4 Cilegon Baru</v>
+        <v>IBT 1 &amp; 2 Suralaya (250 MVA), IBT 4 Cilegon (500 MVA)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>5. Trafo Distribusi / KTT</v>
+        <v>Peralatan (5)</v>
       </c>
       <c r="B6" t="str">
-        <v>trafo_distribusi</v>
+        <v>Trafo Distribusi</v>
       </c>
       <c r="C6" t="str">
-        <v>Dua Cincin Bertaut: Atas Merah (150 kV), Bawah Kuning (20 kV / 70 kV)</v>
+        <v>2 Lingkaran Interlocking (Atas: Merah 150kV, Bawah: Kuning 20kV / 70kV)</v>
       </c>
       <c r="D6" t="str">
-        <v>Transformator penurun tegangan dari transmisi 150 kV ke tegangan menengah 20 kV (atau 70 kV) untuk melayani gardu distribusi &amp; konsumen tegangan tinggi (KTT).</v>
+        <v>Trafo step-down daya di Gardu Induk yang menurunkan tegangan dari 150 kV ke 70 kV atau 20 kV.</v>
       </c>
       <c r="E6" t="str">
-        <v>Trafo KTT SLFDO-1 (78 MVA), KTT PENI (40 MVA), KTT LCI (115 MVA), KTT MTSUI</v>
+        <v>Trafo 150/20 kV GI Distribusi / Feeder KTT</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>6. Busbar (Rel Konduktor)</v>
+        <v>Peralatan (6)</v>
       </c>
       <c r="B7" t="str">
-        <v>busbar</v>
+        <v>Busbar</v>
       </c>
       <c r="C7" t="str">
-        <v>Garis Horisontal Tebal: Biru (500 kV) atau Merah (150 kV)</v>
+        <v>Batang Rel Horizontal Tebal (Cyan/Biru)</v>
       </c>
       <c r="D7" t="str">
-        <v>Rel konduktor pengumpul daya listrik di gardu induk. Dapat diset 'Normal' atau 'Panjang (Wide Busbar)' untuk membentang di atas beberapa bay.</v>
+        <v>Batang konduktor utama di Gardu Induk (GI / GITET) yang mengumpulkan dan membagikan daya listrik.</v>
       </c>
       <c r="E7" t="str">
-        <v>Rel 500 kV Suralaya Baru, Rel 150 kV SRLYA (Wide Busbar), Rel 150 kV CLBRU</v>
+        <v>Suralaya Baru (500 kV), GI SRLYA 150 kV, GI CLBRU 150 kV</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Peralatan (7)</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Beban</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Segitiga Terbalik (∇) Kuning Emas dengan terminal bulatan di atas</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Simbol resmi beban listrik konsumen industri KTT (Konsumen Tegangan Tinggi) atau feeder beban.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>KTT SLFDO-1 (78 MVA), KTT PENI (40 MVA), KTT LCI (115 MVA)</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Peralatan (8)</v>
+      </c>
+      <c r="B9" t="str">
+        <v>PHT (Penghantar)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Kapsul Saluran Transmisi dengan dua bulatan terminal di ujung</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Saluran udara/kabel transmisi tenaga listrik penghubung antar gardu induk.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>PHT Suralaya - Salira Indah, PHT Suralaya - PENI</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
-  <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="35.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="40.83203125" customWidth="1"/>
-    <col min="8" max="8" width="40.83203125" customWidth="1"/>
-    <col min="9" max="9" width="40.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4295,21 +3550,18 @@
         <v>Subsistem</v>
       </c>
       <c r="D1" t="str">
-        <v>Peralatan Terdampak</v>
+        <v>UIT</v>
       </c>
       <c r="E1" t="str">
-        <v>UIT</v>
+        <v>Kondisi / Permasalahan</v>
       </c>
       <c r="F1" t="str">
-        <v>Kondisi / Permasalahan</v>
+        <v>Dampak</v>
       </c>
       <c r="G1" t="str">
-        <v>Dampak</v>
+        <v>Mitigasi</v>
       </c>
       <c r="H1" t="str">
-        <v>Mitigasi</v>
-      </c>
-      <c r="I1" t="str">
         <v>Usulan / Solusi</v>
       </c>
     </row>
@@ -4321,30 +3573,27 @@
         <v>1&amp;2</v>
       </c>
       <c r="C2" t="str">
-        <v>Suralaya - Cilegon</v>
+        <v>Subsistem Suralaya Unit #3 - Suralaya 1,2 – Cilegon 4</v>
       </c>
       <c r="D2" t="str">
-        <v>IBT 1 Suralaya &amp; IBT 2 Suralaya Baru (500/150 kV)</v>
+        <v>JBB</v>
       </c>
       <c r="E2" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="F2" t="str">
         <v>Pembebanan IBT–1,2 Suralaya tidak memenuhi kriteria N–1 saat PLTU Suralaya unit–3 tidak beroperasi dan IBT–4 Cilegon masuk sub sistem Cilegon.</v>
       </c>
-      <c r="G2" t="str" xml:space="preserve">
+      <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Pemeliharaan IBT sulit dilakukan.
 2. Pertumbuhan beban menjadi terhambat.
 3. Terjadi pemadaman apabila trip salah satu IBT di Suralaya.</v>
       </c>
+      <c r="G2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW (Berdasarkan buku DS Tahun 2025).
+2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan total target sebesar 137 MW (Berdasarkan buku DS Tahun 2025).
+3. Pemeliharaan IBT saat beban rendah dan pada saat PLTU Suralaya Unit–3 beroperasi.</v>
+      </c>
       <c r="H2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW.
-2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan target total 137 MW.
-3. Pemeliharaan IBT saat beban rendah dan Unit 3 beroperasi.</v>
-      </c>
-      <c r="I2" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2025/2026.</v>
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2025.</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -4355,27 +3604,26 @@
         <v>2</v>
       </c>
       <c r="C3" t="str">
-        <v>Suralaya - Cilegon</v>
+        <v>Subsistem Suralaya Unit #3 - Suralaya 1,2 – Cilegon 4</v>
       </c>
       <c r="D3" t="str">
-        <v>IBT 4 Cilegon Baru (500/150 kV)</v>
+        <v>JBB</v>
       </c>
       <c r="E3" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="F3" t="str">
         <v>Daya Mampu Pasok IBT Suralaya dan Cilegon tidak sama (IBT #1,2 Suralaya 250 MVA sedangkan IBT #4 Cilegon 500 MVA).</v>
       </c>
+      <c r="F3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Ketidakseimbangan beban antara IBT Suralaya dan IBT Cilegon.
+2. Kondisi N–1–1 (IBT Suralaya dan IBT Cilegon) berdampak overload pada IBT Suralaya yang beroperasi.</v>
+      </c>
       <c r="G3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Ketidakseimbangan beban antara IBT Suralaya dan IBT Cilegon.
-2. Kondisi N–1–1 berdampak overload pada IBT Suralaya yang beroperasi.</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Optimalisasi transfer trip dan defense scheme antar GI.</v>
-      </c>
-      <c r="I3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sudah terpasang DS OLS IBT 1,2 Suralaya dengan target total sebesar 102 MW (Berdasarkan buku DS Tahun 2025).
+2. Rencana penambahan target DS OLS SS Suralaya 1,2 dengan total target sebesar 137 MW (Berdasarkan buku DS Tahun 2025).
+3. Pemeliharaan IBT saat beban rendah dan pada saat PLTU Suralaya Unit–3 beroperasi.</v>
+      </c>
+      <c r="H3" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Pendek :
-Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA.</v>
+Uprating IBT–1 &amp; 2 Suralaya dari 250 MVA menjadi 500 MVA. Berdasarkan RUPTL 2025 – 2034, COD di Tahun 2026.</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -4386,33 +3634,30 @@
         <v>3</v>
       </c>
       <c r="C4" t="str">
-        <v>Suralaya - Cilegon</v>
+        <v>Subsistem Suralaya Unit #3 - Suralaya 1,2 – Cilegon 4</v>
       </c>
       <c r="D4" t="str">
-        <v>Ruas SUTT Suralaya–PENI, Suralaya–MCCI, MCCI–Cilegon, PENI–Mitsui–Cilegon</v>
+        <v>JBB</v>
       </c>
       <c r="E4" t="str">
-        <v>JBB</v>
-      </c>
-      <c r="F4" t="str">
         <v>Ruas Penghantar Suralaya–MCCI–Cilegon dan Suralaya–Peni–Mitsui–Cilegon masih single phi.</v>
       </c>
-      <c r="G4" t="str" xml:space="preserve">
+      <c r="F4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Pemeliharaan Penghantar menjadi sulit dilakukan.
 2. Terjadi pemadaman apabila terdapat gangguan N–1–1.</v>
       </c>
-      <c r="H4" t="str" xml:space="preserve">
+      <c r="G4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Pemeliharaan Penghantar menyesuaikan jadwal dari KTT.
 2. Pengaturan konfigurasi jaringan saat pemeliharaan untuk mengurangi dampak padam.</v>
       </c>
-      <c r="I4" t="str" xml:space="preserve">
+      <c r="H4" t="str" xml:space="preserve">
         <v xml:space="preserve">Jangka Menengah :
 Usulan Double phi pada ruas Suralaya s.d Cilegon Lama (Kajian belum ada). Diusulkan COD Tahun 2030.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sld): tabbed GI panel, canvas UX, deterministic save, template guides
- GI detail panel: tab Informasi/Kerawanan/Aset Terkait/Riwayat with
  real template data in subsystem and system views
- SldSvgCanvas: frozen tier gutter + title, hover-enlarged labels,
  solid label backdrops, light/dark themes on all views
- engine layout: book tier guides, generator stacking and dense-row
  compaction for system backbones
- deterministic save from last parse payload, live counts on save
  button, verify-after-write, bundle hash indicator
- loading overlay with staged progress; drop dead React Flow path
- snapshot versioning + stale auto-drop; honest risk display
- yellow mandatory-column headers in both example templates
- rebuild dist bundle
</commit_message>
<xml_diff>
--- a/peta-kerawanan/dist/template_kerawanan_subsistem_suralaya_cilegon.xlsx
+++ b/peta-kerawanan/dist/template_kerawanan_subsistem_suralaya_cilegon.xlsx
@@ -15,7 +15,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -23,13 +23,26 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -44,8 +57,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,12 +471,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>No Kerawanan</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Nama Penghantar</t>
         </is>
@@ -477,7 +491,7 @@
           <t>Tipe Simbol SLD</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Dari GI</t>
         </is>
@@ -487,12 +501,12 @@
           <t>Tipe Simbol Dari GI</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Tier Dari GI</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Ke GI</t>
         </is>
@@ -502,12 +516,12 @@
           <t>Tipe Simbol Ke GI</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Tier Ke GI</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Tegangan</t>
         </is>
@@ -527,7 +541,7 @@
           <t>Status Operasi</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Tingkat Kerawanan</t>
         </is>
@@ -2468,7 +2482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM25"/>
+  <dimension ref="A1:T25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="18" max="18"/>
@@ -2482,17 +2496,17 @@
           <t>No</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Nama Asset / GI</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Kode Singkatan</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Tipe Simbol SLD</t>
         </is>
@@ -2507,12 +2521,12 @@
           <t>Kapasitas (MVA / MW)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Tier (Mulai 0)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Tegangan</t>
         </is>
@@ -2522,12 +2536,12 @@
           <t>No IBT</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Status Kerawanan</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>No Kerawanan</t>
         </is>
@@ -4457,12 +4471,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>No Kerawanan</t>
         </is>
@@ -4477,7 +4491,7 @@
           <t>UIT</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Kondisi / Permasalahan</t>
         </is>

</xml_diff>

<commit_message>
Koreksi SUTT 500 kV: hub di Suralaya Baru (Suralaya Baru-Cilegon Baru)
</commit_message>
<xml_diff>
--- a/peta-kerawanan/dist/template_kerawanan_subsistem_suralaya_cilegon.xlsx
+++ b/peta-kerawanan/dist/template_kerawanan_subsistem_suralaya_cilegon.xlsx
@@ -2190,7 +2190,7 @@
         <v/>
       </c>
       <c r="C24" t="str">
-        <v>Suralaya - Cilegon Baru</v>
+        <v>Suralaya Baru - Cilegon Baru</v>
       </c>
       <c r="D24" t="str">
         <v>PHT</v>
@@ -2199,7 +2199,7 @@
         <v>PHT</v>
       </c>
       <c r="F24" t="str">
-        <v>Suralaya</v>
+        <v>Suralaya Baru</v>
       </c>
       <c r="G24" t="str">
         <v>Busbar</v>
@@ -2267,7 +2267,7 @@
         <v/>
       </c>
       <c r="C25" t="str">
-        <v>Suralaya - Cilegon Baru</v>
+        <v>Suralaya Baru - Cilegon Baru</v>
       </c>
       <c r="D25" t="str">
         <v>PHT</v>
@@ -2276,7 +2276,7 @@
         <v>PHT</v>
       </c>
       <c r="F25" t="str">
-        <v>Suralaya</v>
+        <v>Suralaya Baru</v>
       </c>
       <c r="G25" t="str">
         <v>Busbar</v>

</xml_diff>